<commit_message>
issue redy to update
</commit_message>
<xml_diff>
--- a/WEB/public/ppe-templates/ppe_template.xlsx
+++ b/WEB/public/ppe-templates/ppe_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeyms\Desktop\ERC-Assets-Management-System\WEB\public\ppe-templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355A93A5-8298-4D34-AC2D-C53C7B324AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D580B871-B900-4CCD-BE45-4320959C658F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB0DB0D6-36BB-43B2-8560-BC35D5F67C71}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t>Property Number</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>Estimated Useful Life (Years)</t>
-  </si>
-  <si>
-    <t>PAR/ITR Number</t>
   </si>
   <si>
     <t>Plantilla Employee ID</t>
@@ -799,7 +796,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
@@ -842,6 +839,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -851,8 +849,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1230,8 +1226,7 @@
     <col min="18" max="18" width="18.7109375" customWidth="1"/>
     <col min="19" max="19" width="19.140625" customWidth="1"/>
     <col min="20" max="20" width="26.28515625" customWidth="1"/>
-    <col min="21" max="21" width="22.140625" customWidth="1"/>
-    <col min="22" max="22" width="23.5703125" customWidth="1"/>
+    <col min="21" max="22" width="16.7109375" customWidth="1"/>
     <col min="23" max="23" width="27.28515625" customWidth="1"/>
     <col min="24" max="24" width="18.7109375" customWidth="1"/>
     <col min="25" max="25" width="14.7109375" customWidth="1"/>
@@ -1239,38 +1234,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="26" t="s">
-        <v>19</v>
+      <c r="A1" s="27" t="s">
+        <v>18</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
       <c r="M1" s="25"/>
-      <c r="N1" s="26" t="s">
-        <v>17</v>
+      <c r="N1" s="27" t="s">
+        <v>16</v>
       </c>
-      <c r="O1" s="27"/>
-      <c r="P1" s="27"/>
-      <c r="Q1" s="27"/>
-      <c r="R1" s="27"/>
-      <c r="S1" s="27"/>
-      <c r="T1" s="28"/>
-      <c r="U1" s="26" t="s">
-        <v>17</v>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="27" t="s">
+        <v>16</v>
       </c>
-      <c r="V1" s="27"/>
-      <c r="W1" s="27"/>
-      <c r="X1" s="27"/>
-      <c r="Y1" s="27"/>
-      <c r="Z1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="29"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1310,46 +1305,46 @@
         <v>11</v>
       </c>
       <c r="M2" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O2" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>22</v>
+      <c r="P2" s="1" t="s">
+        <v>12</v>
       </c>
-      <c r="O2" s="29" t="s">
+      <c r="Q2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="V2" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="1" t="s">
+      <c r="X2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="S2" s="1" t="s">
+      <c r="Z2" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z2" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
@@ -1360,7 +1355,6 @@
       <c r="L3" s="20"/>
       <c r="M3" s="22"/>
       <c r="N3" s="4"/>
-      <c r="O3" s="30"/>
       <c r="R3" s="7"/>
       <c r="T3" s="9"/>
       <c r="U3" s="4"/>
@@ -1375,7 +1369,6 @@
       <c r="L4" s="20"/>
       <c r="M4" s="22"/>
       <c r="N4" s="4"/>
-      <c r="O4" s="30"/>
       <c r="R4" s="7"/>
       <c r="T4" s="9"/>
       <c r="U4" s="4"/>
@@ -1390,7 +1383,6 @@
       <c r="L5" s="20"/>
       <c r="M5" s="22"/>
       <c r="N5" s="4"/>
-      <c r="O5" s="30"/>
       <c r="R5" s="7"/>
       <c r="T5" s="9"/>
       <c r="U5" s="4"/>
@@ -1405,7 +1397,6 @@
       <c r="L6" s="20"/>
       <c r="M6" s="22"/>
       <c r="N6" s="4"/>
-      <c r="O6" s="30"/>
       <c r="R6" s="7"/>
       <c r="T6" s="9"/>
       <c r="U6" s="4"/>
@@ -1420,7 +1411,6 @@
       <c r="L7" s="20"/>
       <c r="M7" s="22"/>
       <c r="N7" s="4"/>
-      <c r="O7" s="30"/>
       <c r="R7" s="7"/>
       <c r="T7" s="9"/>
       <c r="U7" s="4"/>
@@ -1435,7 +1425,6 @@
       <c r="L8" s="20"/>
       <c r="M8" s="22"/>
       <c r="N8" s="4"/>
-      <c r="O8" s="30"/>
       <c r="R8" s="7"/>
       <c r="T8" s="9"/>
       <c r="U8" s="4"/>
@@ -1450,7 +1439,6 @@
       <c r="L9" s="20"/>
       <c r="M9" s="22"/>
       <c r="N9" s="4"/>
-      <c r="O9" s="30"/>
       <c r="R9" s="7"/>
       <c r="T9" s="9"/>
       <c r="U9" s="4"/>
@@ -1464,7 +1452,6 @@
       <c r="L10" s="20"/>
       <c r="M10" s="22"/>
       <c r="N10" s="4"/>
-      <c r="O10" s="30"/>
       <c r="R10" s="7"/>
       <c r="T10" s="9"/>
       <c r="U10" s="4"/>
@@ -1479,7 +1466,6 @@
       <c r="L11" s="20"/>
       <c r="M11" s="22"/>
       <c r="N11" s="4"/>
-      <c r="O11" s="30"/>
       <c r="R11" s="7"/>
       <c r="T11" s="9"/>
       <c r="U11" s="4"/>
@@ -1494,7 +1480,6 @@
       <c r="L12" s="20"/>
       <c r="M12" s="22"/>
       <c r="N12" s="4"/>
-      <c r="O12" s="30"/>
       <c r="R12" s="7"/>
       <c r="T12" s="9"/>
       <c r="U12" s="4"/>
@@ -1508,7 +1493,6 @@
       <c r="L13" s="20"/>
       <c r="M13" s="22"/>
       <c r="N13" s="4"/>
-      <c r="O13" s="30"/>
       <c r="R13" s="7"/>
       <c r="T13" s="9"/>
       <c r="U13" s="4"/>
@@ -1523,7 +1507,6 @@
       <c r="L14" s="20"/>
       <c r="M14" s="22"/>
       <c r="N14" s="4"/>
-      <c r="O14" s="30"/>
       <c r="R14" s="7"/>
       <c r="T14" s="9"/>
       <c r="U14" s="4"/>
@@ -1538,7 +1521,6 @@
       <c r="L15" s="20"/>
       <c r="M15" s="22"/>
       <c r="N15" s="4"/>
-      <c r="O15" s="30"/>
       <c r="R15" s="7"/>
       <c r="T15" s="9"/>
       <c r="U15" s="4"/>
@@ -1552,7 +1534,6 @@
       <c r="L16" s="20"/>
       <c r="M16" s="22"/>
       <c r="N16" s="4"/>
-      <c r="O16" s="30"/>
       <c r="R16" s="7"/>
       <c r="T16" s="9"/>
       <c r="U16" s="4"/>
@@ -1567,7 +1548,6 @@
       <c r="L17" s="20"/>
       <c r="M17" s="22"/>
       <c r="N17" s="4"/>
-      <c r="O17" s="30"/>
       <c r="R17" s="7"/>
       <c r="T17" s="9"/>
       <c r="U17" s="4"/>
@@ -1582,7 +1562,6 @@
       <c r="L18" s="20"/>
       <c r="M18" s="22"/>
       <c r="N18" s="4"/>
-      <c r="O18" s="30"/>
       <c r="R18" s="7"/>
       <c r="T18" s="9"/>
       <c r="U18" s="4"/>
@@ -1596,7 +1575,6 @@
       <c r="L19" s="20"/>
       <c r="M19" s="22"/>
       <c r="N19" s="4"/>
-      <c r="O19" s="30"/>
       <c r="R19" s="7"/>
       <c r="T19" s="9"/>
       <c r="U19" s="4"/>
@@ -1610,7 +1588,6 @@
       <c r="L20" s="20"/>
       <c r="M20" s="22"/>
       <c r="N20" s="4"/>
-      <c r="O20" s="30"/>
       <c r="R20" s="7"/>
       <c r="T20" s="9"/>
       <c r="U20" s="4"/>
@@ -1624,7 +1601,6 @@
       <c r="L21" s="20"/>
       <c r="M21" s="22"/>
       <c r="N21" s="4"/>
-      <c r="O21" s="30"/>
       <c r="R21" s="7"/>
       <c r="T21" s="9"/>
       <c r="U21" s="4"/>
@@ -1639,7 +1615,6 @@
       <c r="L22" s="20"/>
       <c r="M22" s="22"/>
       <c r="N22" s="4"/>
-      <c r="O22" s="30"/>
       <c r="R22" s="7"/>
       <c r="T22" s="9"/>
       <c r="U22" s="4"/>
@@ -1654,7 +1629,6 @@
       <c r="L23" s="20"/>
       <c r="M23" s="22"/>
       <c r="N23" s="4"/>
-      <c r="O23" s="30"/>
       <c r="R23" s="7"/>
       <c r="T23" s="9"/>
       <c r="U23" s="4"/>
@@ -1669,7 +1643,6 @@
       <c r="L24" s="20"/>
       <c r="M24" s="22"/>
       <c r="N24" s="4"/>
-      <c r="O24" s="30"/>
       <c r="R24" s="7"/>
       <c r="T24" s="9"/>
       <c r="U24" s="4"/>
@@ -1684,7 +1657,6 @@
       <c r="L25" s="20"/>
       <c r="M25" s="22"/>
       <c r="N25" s="4"/>
-      <c r="O25" s="30"/>
       <c r="R25" s="7"/>
       <c r="T25" s="9"/>
       <c r="U25" s="4"/>
@@ -1698,7 +1670,6 @@
       <c r="L26" s="20"/>
       <c r="M26" s="22"/>
       <c r="N26" s="4"/>
-      <c r="O26" s="30"/>
       <c r="R26" s="7"/>
       <c r="T26" s="9"/>
       <c r="U26" s="4"/>
@@ -1713,7 +1684,6 @@
       <c r="L27" s="20"/>
       <c r="M27" s="22"/>
       <c r="N27" s="4"/>
-      <c r="O27" s="30"/>
       <c r="R27" s="7"/>
       <c r="T27" s="9"/>
       <c r="U27" s="4"/>
@@ -1728,7 +1698,6 @@
       <c r="L28" s="20"/>
       <c r="M28" s="22"/>
       <c r="N28" s="4"/>
-      <c r="O28" s="30"/>
       <c r="R28" s="7"/>
       <c r="T28" s="9"/>
       <c r="U28" s="4"/>
@@ -1742,7 +1711,6 @@
       <c r="L29" s="20"/>
       <c r="M29" s="22"/>
       <c r="N29" s="4"/>
-      <c r="O29" s="30"/>
       <c r="R29" s="7"/>
       <c r="T29" s="9"/>
       <c r="U29" s="4"/>
@@ -1756,7 +1724,6 @@
       <c r="L30" s="20"/>
       <c r="M30" s="22"/>
       <c r="N30" s="4"/>
-      <c r="O30" s="30"/>
       <c r="R30" s="7"/>
       <c r="T30" s="9"/>
       <c r="U30" s="4"/>
@@ -1771,7 +1738,6 @@
       <c r="L31" s="20"/>
       <c r="M31" s="22"/>
       <c r="N31" s="4"/>
-      <c r="O31" s="30"/>
       <c r="R31" s="7"/>
       <c r="T31" s="9"/>
       <c r="U31" s="4"/>
@@ -1786,7 +1752,6 @@
       <c r="L32" s="20"/>
       <c r="M32" s="22"/>
       <c r="N32" s="4"/>
-      <c r="O32" s="30"/>
       <c r="R32" s="7"/>
       <c r="T32" s="9"/>
       <c r="U32" s="4"/>
@@ -1800,7 +1765,6 @@
       <c r="L33" s="20"/>
       <c r="M33" s="22"/>
       <c r="N33" s="4"/>
-      <c r="O33" s="30"/>
       <c r="R33" s="7"/>
       <c r="T33" s="9"/>
       <c r="U33" s="4"/>
@@ -1814,7 +1778,6 @@
       <c r="L34" s="20"/>
       <c r="M34" s="22"/>
       <c r="N34" s="4"/>
-      <c r="O34" s="30"/>
       <c r="R34" s="7"/>
       <c r="T34" s="9"/>
       <c r="U34" s="4"/>
@@ -1828,7 +1791,6 @@
       <c r="L35" s="20"/>
       <c r="M35" s="22"/>
       <c r="N35" s="4"/>
-      <c r="O35" s="30"/>
       <c r="R35" s="7"/>
       <c r="T35" s="9"/>
       <c r="U35" s="4"/>
@@ -1842,7 +1804,6 @@
       <c r="L36" s="20"/>
       <c r="M36" s="22"/>
       <c r="N36" s="4"/>
-      <c r="O36" s="30"/>
       <c r="R36" s="7"/>
       <c r="T36" s="9"/>
       <c r="U36" s="4"/>
@@ -1856,7 +1817,6 @@
       <c r="L37" s="20"/>
       <c r="M37" s="22"/>
       <c r="N37" s="4"/>
-      <c r="O37" s="30"/>
       <c r="R37" s="7"/>
       <c r="T37" s="9"/>
       <c r="U37" s="4"/>
@@ -1870,7 +1830,6 @@
       <c r="L38" s="20"/>
       <c r="M38" s="22"/>
       <c r="N38" s="4"/>
-      <c r="O38" s="30"/>
       <c r="R38" s="7"/>
       <c r="T38" s="9"/>
       <c r="U38" s="4"/>
@@ -1884,7 +1843,6 @@
       <c r="L39" s="20"/>
       <c r="M39" s="22"/>
       <c r="N39" s="4"/>
-      <c r="O39" s="30"/>
       <c r="R39" s="7"/>
       <c r="T39" s="9"/>
       <c r="U39" s="4"/>
@@ -1898,7 +1856,6 @@
       <c r="L40" s="20"/>
       <c r="M40" s="22"/>
       <c r="N40" s="4"/>
-      <c r="O40" s="30"/>
       <c r="R40" s="7"/>
       <c r="T40" s="9"/>
       <c r="U40" s="4"/>
@@ -1912,7 +1869,6 @@
       <c r="L41" s="20"/>
       <c r="M41" s="22"/>
       <c r="N41" s="4"/>
-      <c r="O41" s="30"/>
       <c r="R41" s="7"/>
       <c r="T41" s="9"/>
       <c r="U41" s="4"/>
@@ -1926,7 +1882,6 @@
       <c r="L42" s="20"/>
       <c r="M42" s="22"/>
       <c r="N42" s="4"/>
-      <c r="O42" s="30"/>
       <c r="R42" s="7"/>
       <c r="T42" s="9"/>
       <c r="U42" s="4"/>
@@ -1940,7 +1895,6 @@
       <c r="L43" s="20"/>
       <c r="M43" s="22"/>
       <c r="N43" s="4"/>
-      <c r="O43" s="30"/>
       <c r="R43" s="7"/>
       <c r="T43" s="9"/>
       <c r="U43" s="4"/>
@@ -1954,7 +1908,6 @@
       <c r="L44" s="20"/>
       <c r="M44" s="22"/>
       <c r="N44" s="4"/>
-      <c r="O44" s="30"/>
       <c r="R44" s="7"/>
       <c r="T44" s="9"/>
       <c r="U44" s="4"/>
@@ -1968,7 +1921,6 @@
       <c r="L45" s="20"/>
       <c r="M45" s="22"/>
       <c r="N45" s="4"/>
-      <c r="O45" s="30"/>
       <c r="R45" s="7"/>
       <c r="T45" s="9"/>
       <c r="U45" s="4"/>
@@ -1982,7 +1934,6 @@
       <c r="L46" s="20"/>
       <c r="M46" s="22"/>
       <c r="N46" s="4"/>
-      <c r="O46" s="30"/>
       <c r="R46" s="7"/>
       <c r="T46" s="9"/>
       <c r="U46" s="4"/>
@@ -1996,7 +1947,6 @@
       <c r="L47" s="20"/>
       <c r="M47" s="22"/>
       <c r="N47" s="4"/>
-      <c r="O47" s="30"/>
       <c r="R47" s="7"/>
       <c r="T47" s="9"/>
       <c r="U47" s="4"/>
@@ -2010,7 +1960,6 @@
       <c r="L48" s="20"/>
       <c r="M48" s="22"/>
       <c r="N48" s="4"/>
-      <c r="O48" s="30"/>
       <c r="R48" s="7"/>
       <c r="T48" s="9"/>
       <c r="U48" s="4"/>
@@ -2024,7 +1973,6 @@
       <c r="L49" s="20"/>
       <c r="M49" s="22"/>
       <c r="N49" s="4"/>
-      <c r="O49" s="30"/>
       <c r="R49" s="7"/>
       <c r="T49" s="9"/>
       <c r="U49" s="4"/>
@@ -2038,7 +1986,6 @@
       <c r="L50" s="20"/>
       <c r="M50" s="22"/>
       <c r="N50" s="4"/>
-      <c r="O50" s="30"/>
       <c r="R50" s="7"/>
       <c r="T50" s="9"/>
       <c r="U50" s="4"/>
@@ -2052,7 +1999,6 @@
       <c r="L51" s="20"/>
       <c r="M51" s="22"/>
       <c r="N51" s="4"/>
-      <c r="O51" s="30"/>
       <c r="R51" s="7"/>
       <c r="T51" s="9"/>
       <c r="U51" s="4"/>
@@ -2066,7 +2012,6 @@
       <c r="L52" s="20"/>
       <c r="M52" s="22"/>
       <c r="N52" s="4"/>
-      <c r="O52" s="30"/>
       <c r="R52" s="7"/>
       <c r="T52" s="9"/>
       <c r="U52" s="4"/>
@@ -2080,7 +2025,6 @@
       <c r="L53" s="20"/>
       <c r="M53" s="22"/>
       <c r="N53" s="4"/>
-      <c r="O53" s="30"/>
       <c r="R53" s="7"/>
       <c r="T53" s="9"/>
       <c r="U53" s="4"/>
@@ -2094,7 +2038,6 @@
       <c r="L54" s="20"/>
       <c r="M54" s="22"/>
       <c r="N54" s="4"/>
-      <c r="O54" s="30"/>
       <c r="R54" s="7"/>
       <c r="T54" s="9"/>
       <c r="U54" s="4"/>
@@ -2108,7 +2051,6 @@
       <c r="L55" s="20"/>
       <c r="M55" s="22"/>
       <c r="N55" s="4"/>
-      <c r="O55" s="30"/>
       <c r="R55" s="7"/>
       <c r="T55" s="9"/>
       <c r="U55" s="4"/>
@@ -2122,7 +2064,6 @@
       <c r="L56" s="20"/>
       <c r="M56" s="22"/>
       <c r="N56" s="4"/>
-      <c r="O56" s="30"/>
       <c r="R56" s="7"/>
       <c r="T56" s="9"/>
       <c r="U56" s="4"/>
@@ -2136,7 +2077,6 @@
       <c r="L57" s="20"/>
       <c r="M57" s="22"/>
       <c r="N57" s="4"/>
-      <c r="O57" s="30"/>
       <c r="R57" s="7"/>
       <c r="T57" s="9"/>
       <c r="U57" s="4"/>
@@ -2150,7 +2090,6 @@
       <c r="L58" s="20"/>
       <c r="M58" s="22"/>
       <c r="N58" s="4"/>
-      <c r="O58" s="30"/>
       <c r="R58" s="7"/>
       <c r="T58" s="9"/>
       <c r="U58" s="4"/>
@@ -2164,7 +2103,6 @@
       <c r="L59" s="20"/>
       <c r="M59" s="22"/>
       <c r="N59" s="4"/>
-      <c r="O59" s="30"/>
       <c r="R59" s="7"/>
       <c r="T59" s="9"/>
       <c r="U59" s="4"/>
@@ -2176,7 +2114,6 @@
       <c r="L60" s="20"/>
       <c r="M60" s="22"/>
       <c r="N60" s="4"/>
-      <c r="O60" s="30"/>
       <c r="T60" s="9"/>
       <c r="U60" s="4"/>
       <c r="Z60" s="9"/>
@@ -2187,7 +2124,6 @@
       <c r="L61" s="20"/>
       <c r="M61" s="22"/>
       <c r="N61" s="4"/>
-      <c r="O61" s="30"/>
       <c r="T61" s="9"/>
       <c r="U61" s="4"/>
       <c r="Z61" s="9"/>
@@ -2198,7 +2134,6 @@
       <c r="L62" s="20"/>
       <c r="M62" s="22"/>
       <c r="N62" s="4"/>
-      <c r="O62" s="30"/>
       <c r="T62" s="9"/>
       <c r="U62" s="4"/>
       <c r="Z62" s="9"/>
@@ -2209,7 +2144,6 @@
       <c r="L63" s="20"/>
       <c r="M63" s="22"/>
       <c r="N63" s="4"/>
-      <c r="O63" s="30"/>
       <c r="T63" s="9"/>
       <c r="U63" s="4"/>
       <c r="Z63" s="9"/>
@@ -2220,7 +2154,6 @@
       <c r="L64" s="20"/>
       <c r="M64" s="22"/>
       <c r="N64" s="4"/>
-      <c r="O64" s="30"/>
       <c r="T64" s="9"/>
       <c r="U64" s="4"/>
       <c r="Z64" s="9"/>
@@ -2231,7 +2164,6 @@
       <c r="L65" s="20"/>
       <c r="M65" s="22"/>
       <c r="N65" s="4"/>
-      <c r="O65" s="30"/>
       <c r="T65" s="9"/>
       <c r="U65" s="4"/>
       <c r="Z65" s="9"/>
@@ -2242,7 +2174,6 @@
       <c r="L66" s="20"/>
       <c r="M66" s="22"/>
       <c r="N66" s="4"/>
-      <c r="O66" s="30"/>
       <c r="T66" s="9"/>
       <c r="U66" s="4"/>
       <c r="Z66" s="9"/>
@@ -2253,7 +2184,6 @@
       <c r="L67" s="20"/>
       <c r="M67" s="22"/>
       <c r="N67" s="4"/>
-      <c r="O67" s="30"/>
       <c r="T67" s="9"/>
       <c r="U67" s="4"/>
       <c r="Z67" s="9"/>
@@ -2264,7 +2194,6 @@
       <c r="L68" s="20"/>
       <c r="M68" s="22"/>
       <c r="N68" s="4"/>
-      <c r="O68" s="30"/>
       <c r="T68" s="9"/>
       <c r="U68" s="4"/>
       <c r="Z68" s="9"/>
@@ -2275,7 +2204,6 @@
       <c r="L69" s="20"/>
       <c r="M69" s="22"/>
       <c r="N69" s="4"/>
-      <c r="O69" s="30"/>
       <c r="T69" s="9"/>
       <c r="U69" s="4"/>
       <c r="Z69" s="9"/>
@@ -2286,7 +2214,6 @@
       <c r="L70" s="20"/>
       <c r="M70" s="22"/>
       <c r="N70" s="4"/>
-      <c r="O70" s="30"/>
       <c r="T70" s="9"/>
       <c r="U70" s="4"/>
       <c r="Z70" s="9"/>
@@ -2297,7 +2224,6 @@
       <c r="L71" s="20"/>
       <c r="M71" s="22"/>
       <c r="N71" s="4"/>
-      <c r="O71" s="30"/>
       <c r="T71" s="9"/>
       <c r="U71" s="4"/>
       <c r="Z71" s="9"/>
@@ -2308,7 +2234,6 @@
       <c r="L72" s="20"/>
       <c r="M72" s="22"/>
       <c r="N72" s="4"/>
-      <c r="O72" s="30"/>
       <c r="T72" s="9"/>
       <c r="U72" s="4"/>
       <c r="Z72" s="9"/>
@@ -2319,7 +2244,6 @@
       <c r="L73" s="20"/>
       <c r="M73" s="22"/>
       <c r="N73" s="4"/>
-      <c r="O73" s="30"/>
       <c r="T73" s="9"/>
       <c r="U73" s="4"/>
       <c r="Z73" s="9"/>
@@ -2330,7 +2254,6 @@
       <c r="L74" s="20"/>
       <c r="M74" s="22"/>
       <c r="N74" s="4"/>
-      <c r="O74" s="30"/>
       <c r="T74" s="9"/>
       <c r="U74" s="4"/>
       <c r="Z74" s="9"/>
@@ -2341,7 +2264,6 @@
       <c r="L75" s="20"/>
       <c r="M75" s="22"/>
       <c r="N75" s="4"/>
-      <c r="O75" s="30"/>
       <c r="T75" s="9"/>
       <c r="U75" s="4"/>
       <c r="Z75" s="9"/>
@@ -2352,7 +2274,6 @@
       <c r="L76" s="20"/>
       <c r="M76" s="22"/>
       <c r="N76" s="4"/>
-      <c r="O76" s="30"/>
       <c r="T76" s="9"/>
       <c r="U76" s="4"/>
       <c r="Z76" s="9"/>
@@ -2363,7 +2284,6 @@
       <c r="L77" s="20"/>
       <c r="M77" s="22"/>
       <c r="N77" s="4"/>
-      <c r="O77" s="30"/>
       <c r="T77" s="9"/>
       <c r="U77" s="4"/>
       <c r="Z77" s="9"/>
@@ -2374,7 +2294,6 @@
       <c r="L78" s="20"/>
       <c r="M78" s="22"/>
       <c r="N78" s="4"/>
-      <c r="O78" s="30"/>
       <c r="T78" s="9"/>
       <c r="U78" s="4"/>
       <c r="Z78" s="9"/>
@@ -2385,7 +2304,6 @@
       <c r="L79" s="20"/>
       <c r="M79" s="22"/>
       <c r="N79" s="4"/>
-      <c r="O79" s="30"/>
       <c r="T79" s="9"/>
       <c r="U79" s="4"/>
       <c r="Z79" s="9"/>
@@ -2396,7 +2314,6 @@
       <c r="L80" s="20"/>
       <c r="M80" s="22"/>
       <c r="N80" s="4"/>
-      <c r="O80" s="30"/>
       <c r="T80" s="9"/>
       <c r="U80" s="4"/>
       <c r="Z80" s="9"/>
@@ -2407,7 +2324,6 @@
       <c r="L81" s="20"/>
       <c r="M81" s="22"/>
       <c r="N81" s="4"/>
-      <c r="O81" s="30"/>
       <c r="T81" s="9"/>
       <c r="U81" s="4"/>
       <c r="Z81" s="9"/>
@@ -2418,7 +2334,6 @@
       <c r="L82" s="20"/>
       <c r="M82" s="22"/>
       <c r="N82" s="4"/>
-      <c r="O82" s="30"/>
       <c r="T82" s="9"/>
       <c r="U82" s="4"/>
       <c r="Z82" s="9"/>
@@ -2429,7 +2344,6 @@
       <c r="L83" s="20"/>
       <c r="M83" s="22"/>
       <c r="N83" s="4"/>
-      <c r="O83" s="30"/>
       <c r="T83" s="9"/>
       <c r="U83" s="4"/>
       <c r="Z83" s="9"/>
@@ -2440,7 +2354,6 @@
       <c r="L84" s="20"/>
       <c r="M84" s="22"/>
       <c r="N84" s="4"/>
-      <c r="O84" s="30"/>
       <c r="T84" s="9"/>
       <c r="U84" s="4"/>
       <c r="Z84" s="9"/>
@@ -2451,7 +2364,6 @@
       <c r="L85" s="20"/>
       <c r="M85" s="22"/>
       <c r="N85" s="4"/>
-      <c r="O85" s="30"/>
       <c r="T85" s="9"/>
       <c r="U85" s="4"/>
       <c r="Z85" s="9"/>
@@ -2462,7 +2374,6 @@
       <c r="L86" s="20"/>
       <c r="M86" s="22"/>
       <c r="N86" s="4"/>
-      <c r="O86" s="30"/>
       <c r="T86" s="9"/>
       <c r="U86" s="4"/>
       <c r="Z86" s="9"/>
@@ -2473,7 +2384,6 @@
       <c r="L87" s="20"/>
       <c r="M87" s="22"/>
       <c r="N87" s="4"/>
-      <c r="O87" s="30"/>
       <c r="T87" s="9"/>
       <c r="U87" s="4"/>
       <c r="Z87" s="9"/>
@@ -2484,7 +2394,6 @@
       <c r="L88" s="20"/>
       <c r="M88" s="22"/>
       <c r="N88" s="4"/>
-      <c r="O88" s="30"/>
       <c r="T88" s="9"/>
       <c r="U88" s="4"/>
       <c r="Z88" s="9"/>
@@ -2495,7 +2404,6 @@
       <c r="L89" s="20"/>
       <c r="M89" s="22"/>
       <c r="N89" s="4"/>
-      <c r="O89" s="30"/>
       <c r="T89" s="9"/>
       <c r="U89" s="4"/>
       <c r="Z89" s="9"/>
@@ -2506,7 +2414,6 @@
       <c r="L90" s="20"/>
       <c r="M90" s="22"/>
       <c r="N90" s="4"/>
-      <c r="O90" s="30"/>
       <c r="T90" s="9"/>
       <c r="U90" s="4"/>
       <c r="Z90" s="9"/>
@@ -2517,7 +2424,6 @@
       <c r="L91" s="20"/>
       <c r="M91" s="22"/>
       <c r="N91" s="4"/>
-      <c r="O91" s="30"/>
       <c r="T91" s="9"/>
       <c r="U91" s="4"/>
       <c r="Z91" s="9"/>
@@ -2528,7 +2434,6 @@
       <c r="L92" s="20"/>
       <c r="M92" s="22"/>
       <c r="N92" s="4"/>
-      <c r="O92" s="30"/>
       <c r="T92" s="9"/>
       <c r="U92" s="4"/>
       <c r="Z92" s="9"/>
@@ -2539,7 +2444,6 @@
       <c r="L93" s="20"/>
       <c r="M93" s="22"/>
       <c r="N93" s="4"/>
-      <c r="O93" s="30"/>
       <c r="T93" s="9"/>
       <c r="U93" s="4"/>
       <c r="Z93" s="9"/>
@@ -2550,7 +2454,6 @@
       <c r="L94" s="20"/>
       <c r="M94" s="22"/>
       <c r="N94" s="4"/>
-      <c r="O94" s="30"/>
       <c r="T94" s="9"/>
       <c r="U94" s="4"/>
       <c r="Z94" s="9"/>
@@ -2561,7 +2464,6 @@
       <c r="L95" s="20"/>
       <c r="M95" s="22"/>
       <c r="N95" s="4"/>
-      <c r="O95" s="30"/>
       <c r="T95" s="9"/>
       <c r="U95" s="4"/>
       <c r="Z95" s="9"/>
@@ -2572,7 +2474,6 @@
       <c r="L96" s="20"/>
       <c r="M96" s="22"/>
       <c r="N96" s="4"/>
-      <c r="O96" s="30"/>
       <c r="T96" s="9"/>
       <c r="U96" s="4"/>
       <c r="Z96" s="9"/>
@@ -2583,7 +2484,6 @@
       <c r="L97" s="20"/>
       <c r="M97" s="22"/>
       <c r="N97" s="4"/>
-      <c r="O97" s="30"/>
       <c r="T97" s="9"/>
       <c r="U97" s="4"/>
       <c r="Z97" s="9"/>
@@ -2594,7 +2494,6 @@
       <c r="L98" s="20"/>
       <c r="M98" s="22"/>
       <c r="N98" s="4"/>
-      <c r="O98" s="30"/>
       <c r="T98" s="9"/>
       <c r="U98" s="4"/>
       <c r="Z98" s="9"/>
@@ -2605,7 +2504,6 @@
       <c r="L99" s="20"/>
       <c r="M99" s="22"/>
       <c r="N99" s="4"/>
-      <c r="O99" s="30"/>
       <c r="T99" s="9"/>
       <c r="U99" s="4"/>
       <c r="Z99" s="9"/>
@@ -2616,7 +2514,6 @@
       <c r="L100" s="20"/>
       <c r="M100" s="22"/>
       <c r="N100" s="4"/>
-      <c r="O100" s="30"/>
       <c r="T100" s="9"/>
       <c r="U100" s="4"/>
       <c r="Z100" s="9"/>
@@ -2627,7 +2524,6 @@
       <c r="L101" s="20"/>
       <c r="M101" s="22"/>
       <c r="N101" s="4"/>
-      <c r="O101" s="30"/>
       <c r="T101" s="9"/>
       <c r="U101" s="4"/>
       <c r="Z101" s="9"/>
@@ -2638,7 +2534,6 @@
       <c r="L102" s="20"/>
       <c r="M102" s="22"/>
       <c r="N102" s="4"/>
-      <c r="O102" s="30"/>
       <c r="T102" s="9"/>
       <c r="U102" s="4"/>
       <c r="Z102" s="9"/>
@@ -2649,7 +2544,6 @@
       <c r="L103" s="20"/>
       <c r="M103" s="22"/>
       <c r="N103" s="4"/>
-      <c r="O103" s="30"/>
       <c r="T103" s="9"/>
       <c r="U103" s="4"/>
       <c r="Z103" s="9"/>
@@ -2660,7 +2554,6 @@
       <c r="L104" s="20"/>
       <c r="M104" s="22"/>
       <c r="N104" s="4"/>
-      <c r="O104" s="30"/>
       <c r="T104" s="9"/>
       <c r="U104" s="4"/>
       <c r="Z104" s="9"/>
@@ -2671,7 +2564,6 @@
       <c r="L105" s="20"/>
       <c r="M105" s="22"/>
       <c r="N105" s="4"/>
-      <c r="O105" s="30"/>
       <c r="T105" s="9"/>
       <c r="U105" s="4"/>
       <c r="Z105" s="9"/>
@@ -2682,7 +2574,6 @@
       <c r="L106" s="20"/>
       <c r="M106" s="22"/>
       <c r="N106" s="4"/>
-      <c r="O106" s="30"/>
       <c r="T106" s="9"/>
       <c r="U106" s="4"/>
       <c r="Z106" s="9"/>
@@ -2693,7 +2584,6 @@
       <c r="L107" s="20"/>
       <c r="M107" s="22"/>
       <c r="N107" s="4"/>
-      <c r="O107" s="30"/>
       <c r="T107" s="9"/>
       <c r="U107" s="4"/>
       <c r="Z107" s="9"/>
@@ -2704,7 +2594,6 @@
       <c r="L108" s="20"/>
       <c r="M108" s="22"/>
       <c r="N108" s="4"/>
-      <c r="O108" s="30"/>
       <c r="T108" s="9"/>
       <c r="U108" s="4"/>
       <c r="Z108" s="9"/>
@@ -2715,7 +2604,6 @@
       <c r="L109" s="20"/>
       <c r="M109" s="22"/>
       <c r="N109" s="4"/>
-      <c r="O109" s="30"/>
       <c r="T109" s="9"/>
       <c r="U109" s="4"/>
       <c r="Z109" s="9"/>
@@ -2726,7 +2614,6 @@
       <c r="L110" s="20"/>
       <c r="M110" s="22"/>
       <c r="N110" s="4"/>
-      <c r="O110" s="30"/>
       <c r="T110" s="9"/>
       <c r="U110" s="4"/>
       <c r="Z110" s="9"/>
@@ -2737,7 +2624,6 @@
       <c r="L111" s="20"/>
       <c r="M111" s="22"/>
       <c r="N111" s="4"/>
-      <c r="O111" s="30"/>
       <c r="T111" s="9"/>
       <c r="U111" s="4"/>
       <c r="Z111" s="9"/>
@@ -2748,7 +2634,6 @@
       <c r="L112" s="20"/>
       <c r="M112" s="22"/>
       <c r="N112" s="4"/>
-      <c r="O112" s="30"/>
       <c r="T112" s="9"/>
       <c r="U112" s="4"/>
       <c r="Z112" s="9"/>
@@ -2759,7 +2644,6 @@
       <c r="L113" s="20"/>
       <c r="M113" s="22"/>
       <c r="N113" s="4"/>
-      <c r="O113" s="30"/>
       <c r="T113" s="9"/>
       <c r="U113" s="4"/>
       <c r="Z113" s="9"/>
@@ -2770,7 +2654,6 @@
       <c r="L114" s="20"/>
       <c r="M114" s="22"/>
       <c r="N114" s="4"/>
-      <c r="O114" s="30"/>
       <c r="T114" s="9"/>
       <c r="U114" s="4"/>
       <c r="Z114" s="9"/>
@@ -2781,7 +2664,6 @@
       <c r="L115" s="20"/>
       <c r="M115" s="22"/>
       <c r="N115" s="4"/>
-      <c r="O115" s="30"/>
       <c r="T115" s="9"/>
       <c r="U115" s="4"/>
       <c r="Z115" s="9"/>
@@ -2792,7 +2674,6 @@
       <c r="L116" s="20"/>
       <c r="M116" s="22"/>
       <c r="N116" s="4"/>
-      <c r="O116" s="30"/>
       <c r="T116" s="9"/>
       <c r="U116" s="4"/>
       <c r="Z116" s="9"/>
@@ -2803,7 +2684,6 @@
       <c r="L117" s="20"/>
       <c r="M117" s="22"/>
       <c r="N117" s="4"/>
-      <c r="O117" s="30"/>
       <c r="T117" s="9"/>
       <c r="U117" s="4"/>
       <c r="Z117" s="9"/>
@@ -2814,7 +2694,6 @@
       <c r="L118" s="20"/>
       <c r="M118" s="22"/>
       <c r="N118" s="4"/>
-      <c r="O118" s="30"/>
       <c r="T118" s="9"/>
       <c r="U118" s="4"/>
       <c r="Z118" s="9"/>
@@ -2825,7 +2704,6 @@
       <c r="L119" s="20"/>
       <c r="M119" s="22"/>
       <c r="N119" s="4"/>
-      <c r="O119" s="30"/>
       <c r="T119" s="9"/>
       <c r="U119" s="4"/>
       <c r="Z119" s="9"/>
@@ -2836,7 +2714,6 @@
       <c r="L120" s="20"/>
       <c r="M120" s="22"/>
       <c r="N120" s="4"/>
-      <c r="O120" s="30"/>
       <c r="T120" s="9"/>
       <c r="U120" s="4"/>
       <c r="Z120" s="9"/>
@@ -2847,7 +2724,6 @@
       <c r="L121" s="20"/>
       <c r="M121" s="22"/>
       <c r="N121" s="4"/>
-      <c r="O121" s="30"/>
       <c r="T121" s="9"/>
       <c r="U121" s="4"/>
       <c r="Z121" s="9"/>
@@ -2858,7 +2734,6 @@
       <c r="L122" s="20"/>
       <c r="M122" s="22"/>
       <c r="N122" s="4"/>
-      <c r="O122" s="30"/>
       <c r="T122" s="9"/>
       <c r="U122" s="4"/>
       <c r="Z122" s="9"/>
@@ -2869,7 +2744,6 @@
       <c r="L123" s="20"/>
       <c r="M123" s="22"/>
       <c r="N123" s="4"/>
-      <c r="O123" s="30"/>
       <c r="T123" s="9"/>
       <c r="U123" s="4"/>
       <c r="Z123" s="9"/>
@@ -2880,7 +2754,6 @@
       <c r="L124" s="20"/>
       <c r="M124" s="22"/>
       <c r="N124" s="4"/>
-      <c r="O124" s="30"/>
       <c r="T124" s="9"/>
       <c r="U124" s="4"/>
       <c r="Z124" s="9"/>
@@ -2891,7 +2764,6 @@
       <c r="L125" s="20"/>
       <c r="M125" s="22"/>
       <c r="N125" s="4"/>
-      <c r="O125" s="30"/>
       <c r="T125" s="9"/>
       <c r="U125" s="4"/>
       <c r="Z125" s="9"/>
@@ -2902,7 +2774,6 @@
       <c r="L126" s="20"/>
       <c r="M126" s="22"/>
       <c r="N126" s="4"/>
-      <c r="O126" s="30"/>
       <c r="T126" s="9"/>
       <c r="U126" s="4"/>
       <c r="Z126" s="9"/>
@@ -2913,7 +2784,6 @@
       <c r="L127" s="20"/>
       <c r="M127" s="22"/>
       <c r="N127" s="4"/>
-      <c r="O127" s="30"/>
       <c r="T127" s="9"/>
       <c r="U127" s="4"/>
       <c r="Z127" s="9"/>
@@ -2924,7 +2794,6 @@
       <c r="L128" s="20"/>
       <c r="M128" s="22"/>
       <c r="N128" s="4"/>
-      <c r="O128" s="30"/>
       <c r="T128" s="9"/>
       <c r="U128" s="4"/>
       <c r="Z128" s="9"/>
@@ -2935,7 +2804,6 @@
       <c r="L129" s="20"/>
       <c r="M129" s="22"/>
       <c r="N129" s="4"/>
-      <c r="O129" s="30"/>
       <c r="T129" s="9"/>
       <c r="U129" s="4"/>
       <c r="Z129" s="9"/>
@@ -2946,7 +2814,6 @@
       <c r="L130" s="20"/>
       <c r="M130" s="22"/>
       <c r="N130" s="4"/>
-      <c r="O130" s="30"/>
       <c r="T130" s="9"/>
       <c r="U130" s="4"/>
       <c r="Z130" s="9"/>
@@ -2957,7 +2824,6 @@
       <c r="L131" s="20"/>
       <c r="M131" s="22"/>
       <c r="N131" s="4"/>
-      <c r="O131" s="30"/>
       <c r="T131" s="9"/>
       <c r="U131" s="4"/>
       <c r="Z131" s="9"/>
@@ -2968,7 +2834,6 @@
       <c r="L132" s="20"/>
       <c r="M132" s="22"/>
       <c r="N132" s="4"/>
-      <c r="O132" s="30"/>
       <c r="T132" s="9"/>
       <c r="U132" s="4"/>
       <c r="Z132" s="9"/>
@@ -2979,7 +2844,6 @@
       <c r="L133" s="20"/>
       <c r="M133" s="22"/>
       <c r="N133" s="4"/>
-      <c r="O133" s="30"/>
       <c r="T133" s="9"/>
       <c r="U133" s="4"/>
       <c r="Z133" s="9"/>
@@ -2990,7 +2854,6 @@
       <c r="L134" s="20"/>
       <c r="M134" s="22"/>
       <c r="N134" s="4"/>
-      <c r="O134" s="30"/>
       <c r="T134" s="9"/>
       <c r="U134" s="4"/>
       <c r="Z134" s="9"/>
@@ -3001,7 +2864,6 @@
       <c r="L135" s="20"/>
       <c r="M135" s="22"/>
       <c r="N135" s="4"/>
-      <c r="O135" s="30"/>
       <c r="T135" s="9"/>
       <c r="U135" s="4"/>
       <c r="Z135" s="9"/>
@@ -3012,7 +2874,6 @@
       <c r="L136" s="20"/>
       <c r="M136" s="22"/>
       <c r="N136" s="4"/>
-      <c r="O136" s="30"/>
       <c r="T136" s="9"/>
       <c r="U136" s="4"/>
       <c r="Z136" s="9"/>
@@ -3023,7 +2884,6 @@
       <c r="L137" s="20"/>
       <c r="M137" s="22"/>
       <c r="N137" s="4"/>
-      <c r="O137" s="30"/>
       <c r="T137" s="9"/>
       <c r="U137" s="4"/>
       <c r="Z137" s="9"/>
@@ -3034,7 +2894,6 @@
       <c r="L138" s="20"/>
       <c r="M138" s="22"/>
       <c r="N138" s="4"/>
-      <c r="O138" s="30"/>
       <c r="T138" s="9"/>
       <c r="U138" s="4"/>
       <c r="Z138" s="9"/>
@@ -3045,7 +2904,6 @@
       <c r="L139" s="20"/>
       <c r="M139" s="22"/>
       <c r="N139" s="4"/>
-      <c r="O139" s="30"/>
       <c r="T139" s="9"/>
       <c r="U139" s="4"/>
       <c r="Z139" s="9"/>
@@ -3056,7 +2914,6 @@
       <c r="L140" s="20"/>
       <c r="M140" s="22"/>
       <c r="N140" s="4"/>
-      <c r="O140" s="30"/>
       <c r="T140" s="9"/>
       <c r="U140" s="4"/>
       <c r="Z140" s="9"/>
@@ -3067,7 +2924,6 @@
       <c r="L141" s="20"/>
       <c r="M141" s="22"/>
       <c r="N141" s="4"/>
-      <c r="O141" s="30"/>
       <c r="T141" s="9"/>
       <c r="U141" s="4"/>
       <c r="Z141" s="9"/>
@@ -3078,7 +2934,6 @@
       <c r="L142" s="20"/>
       <c r="M142" s="22"/>
       <c r="N142" s="4"/>
-      <c r="O142" s="30"/>
       <c r="T142" s="9"/>
       <c r="U142" s="4"/>
       <c r="Z142" s="9"/>
@@ -3089,7 +2944,6 @@
       <c r="L143" s="20"/>
       <c r="M143" s="22"/>
       <c r="N143" s="4"/>
-      <c r="O143" s="30"/>
       <c r="T143" s="9"/>
       <c r="U143" s="4"/>
       <c r="Z143" s="9"/>
@@ -3100,7 +2954,6 @@
       <c r="L144" s="20"/>
       <c r="M144" s="22"/>
       <c r="N144" s="4"/>
-      <c r="O144" s="30"/>
       <c r="T144" s="9"/>
       <c r="U144" s="4"/>
       <c r="Z144" s="9"/>
@@ -3111,7 +2964,6 @@
       <c r="L145" s="20"/>
       <c r="M145" s="22"/>
       <c r="N145" s="4"/>
-      <c r="O145" s="30"/>
       <c r="T145" s="9"/>
       <c r="U145" s="4"/>
       <c r="Z145" s="9"/>
@@ -3122,7 +2974,6 @@
       <c r="L146" s="20"/>
       <c r="M146" s="22"/>
       <c r="N146" s="4"/>
-      <c r="O146" s="30"/>
       <c r="T146" s="9"/>
       <c r="U146" s="4"/>
       <c r="Z146" s="9"/>
@@ -3133,7 +2984,6 @@
       <c r="L147" s="20"/>
       <c r="M147" s="22"/>
       <c r="N147" s="4"/>
-      <c r="O147" s="30"/>
       <c r="T147" s="9"/>
       <c r="U147" s="4"/>
       <c r="Z147" s="9"/>
@@ -3144,7 +2994,6 @@
       <c r="L148" s="20"/>
       <c r="M148" s="22"/>
       <c r="N148" s="4"/>
-      <c r="O148" s="30"/>
       <c r="T148" s="9"/>
       <c r="U148" s="4"/>
       <c r="Z148" s="9"/>
@@ -3155,7 +3004,6 @@
       <c r="L149" s="20"/>
       <c r="M149" s="22"/>
       <c r="N149" s="4"/>
-      <c r="O149" s="30"/>
       <c r="T149" s="9"/>
       <c r="U149" s="4"/>
       <c r="Z149" s="9"/>
@@ -3166,7 +3014,6 @@
       <c r="L150" s="20"/>
       <c r="M150" s="22"/>
       <c r="N150" s="4"/>
-      <c r="O150" s="30"/>
       <c r="T150" s="9"/>
       <c r="U150" s="4"/>
       <c r="Z150" s="9"/>
@@ -3177,7 +3024,6 @@
       <c r="L151" s="20"/>
       <c r="M151" s="22"/>
       <c r="N151" s="4"/>
-      <c r="O151" s="30"/>
       <c r="T151" s="9"/>
       <c r="U151" s="4"/>
       <c r="Z151" s="9"/>
@@ -3188,7 +3034,6 @@
       <c r="L152" s="20"/>
       <c r="M152" s="22"/>
       <c r="N152" s="4"/>
-      <c r="O152" s="30"/>
       <c r="T152" s="9"/>
       <c r="U152" s="4"/>
       <c r="Z152" s="9"/>
@@ -3199,7 +3044,6 @@
       <c r="L153" s="20"/>
       <c r="M153" s="22"/>
       <c r="N153" s="4"/>
-      <c r="O153" s="30"/>
       <c r="T153" s="9"/>
       <c r="U153" s="4"/>
       <c r="Z153" s="9"/>
@@ -3210,7 +3054,6 @@
       <c r="L154" s="20"/>
       <c r="M154" s="22"/>
       <c r="N154" s="4"/>
-      <c r="O154" s="30"/>
       <c r="T154" s="9"/>
       <c r="U154" s="4"/>
       <c r="Z154" s="9"/>
@@ -3221,7 +3064,6 @@
       <c r="L155" s="20"/>
       <c r="M155" s="22"/>
       <c r="N155" s="4"/>
-      <c r="O155" s="30"/>
       <c r="T155" s="9"/>
       <c r="U155" s="4"/>
       <c r="Z155" s="9"/>
@@ -3232,7 +3074,6 @@
       <c r="L156" s="20"/>
       <c r="M156" s="22"/>
       <c r="N156" s="4"/>
-      <c r="O156" s="30"/>
       <c r="T156" s="9"/>
       <c r="U156" s="4"/>
       <c r="Z156" s="9"/>
@@ -3243,7 +3084,6 @@
       <c r="L157" s="20"/>
       <c r="M157" s="22"/>
       <c r="N157" s="4"/>
-      <c r="O157" s="30"/>
       <c r="T157" s="9"/>
       <c r="U157" s="4"/>
       <c r="Z157" s="9"/>
@@ -3254,7 +3094,6 @@
       <c r="L158" s="20"/>
       <c r="M158" s="22"/>
       <c r="N158" s="4"/>
-      <c r="O158" s="30"/>
       <c r="T158" s="9"/>
       <c r="U158" s="4"/>
       <c r="Z158" s="9"/>
@@ -3265,7 +3104,6 @@
       <c r="L159" s="20"/>
       <c r="M159" s="22"/>
       <c r="N159" s="4"/>
-      <c r="O159" s="30"/>
       <c r="T159" s="9"/>
       <c r="U159" s="4"/>
       <c r="Z159" s="9"/>
@@ -3276,7 +3114,6 @@
       <c r="L160" s="20"/>
       <c r="M160" s="22"/>
       <c r="N160" s="4"/>
-      <c r="O160" s="30"/>
       <c r="T160" s="9"/>
       <c r="U160" s="4"/>
       <c r="Z160" s="9"/>
@@ -3287,7 +3124,6 @@
       <c r="L161" s="20"/>
       <c r="M161" s="22"/>
       <c r="N161" s="4"/>
-      <c r="O161" s="30"/>
       <c r="T161" s="9"/>
       <c r="U161" s="4"/>
       <c r="Z161" s="9"/>
@@ -3298,7 +3134,6 @@
       <c r="L162" s="20"/>
       <c r="M162" s="22"/>
       <c r="N162" s="4"/>
-      <c r="O162" s="30"/>
       <c r="T162" s="9"/>
       <c r="U162" s="4"/>
       <c r="Z162" s="9"/>
@@ -3309,7 +3144,6 @@
       <c r="L163" s="20"/>
       <c r="M163" s="22"/>
       <c r="N163" s="4"/>
-      <c r="O163" s="30"/>
       <c r="T163" s="9"/>
       <c r="U163" s="4"/>
       <c r="Z163" s="9"/>
@@ -3320,7 +3154,6 @@
       <c r="L164" s="20"/>
       <c r="M164" s="22"/>
       <c r="N164" s="4"/>
-      <c r="O164" s="30"/>
       <c r="T164" s="9"/>
       <c r="U164" s="4"/>
       <c r="Z164" s="9"/>
@@ -3331,7 +3164,6 @@
       <c r="L165" s="20"/>
       <c r="M165" s="22"/>
       <c r="N165" s="4"/>
-      <c r="O165" s="30"/>
       <c r="T165" s="9"/>
       <c r="U165" s="4"/>
       <c r="Z165" s="9"/>
@@ -3342,7 +3174,6 @@
       <c r="L166" s="20"/>
       <c r="M166" s="22"/>
       <c r="N166" s="4"/>
-      <c r="O166" s="30"/>
       <c r="T166" s="9"/>
       <c r="U166" s="4"/>
       <c r="Z166" s="9"/>
@@ -3353,7 +3184,6 @@
       <c r="L167" s="20"/>
       <c r="M167" s="22"/>
       <c r="N167" s="4"/>
-      <c r="O167" s="30"/>
       <c r="T167" s="9"/>
       <c r="U167" s="4"/>
       <c r="Z167" s="9"/>
@@ -3364,7 +3194,6 @@
       <c r="L168" s="20"/>
       <c r="M168" s="22"/>
       <c r="N168" s="4"/>
-      <c r="O168" s="30"/>
       <c r="T168" s="9"/>
       <c r="U168" s="4"/>
       <c r="Z168" s="9"/>
@@ -3375,7 +3204,6 @@
       <c r="L169" s="20"/>
       <c r="M169" s="22"/>
       <c r="N169" s="4"/>
-      <c r="O169" s="30"/>
       <c r="T169" s="9"/>
       <c r="U169" s="4"/>
       <c r="Z169" s="9"/>
@@ -3386,7 +3214,6 @@
       <c r="L170" s="20"/>
       <c r="M170" s="22"/>
       <c r="N170" s="4"/>
-      <c r="O170" s="30"/>
       <c r="T170" s="9"/>
       <c r="U170" s="4"/>
       <c r="Z170" s="9"/>
@@ -3397,7 +3224,6 @@
       <c r="L171" s="20"/>
       <c r="M171" s="22"/>
       <c r="N171" s="4"/>
-      <c r="O171" s="30"/>
       <c r="T171" s="9"/>
       <c r="U171" s="4"/>
       <c r="Z171" s="9"/>
@@ -3408,7 +3234,6 @@
       <c r="L172" s="20"/>
       <c r="M172" s="22"/>
       <c r="N172" s="4"/>
-      <c r="O172" s="30"/>
       <c r="T172" s="9"/>
       <c r="U172" s="4"/>
       <c r="Z172" s="9"/>
@@ -3419,7 +3244,6 @@
       <c r="L173" s="20"/>
       <c r="M173" s="22"/>
       <c r="N173" s="4"/>
-      <c r="O173" s="30"/>
       <c r="T173" s="9"/>
       <c r="U173" s="4"/>
       <c r="Z173" s="9"/>
@@ -3430,7 +3254,6 @@
       <c r="L174" s="20"/>
       <c r="M174" s="22"/>
       <c r="N174" s="4"/>
-      <c r="O174" s="30"/>
       <c r="T174" s="9"/>
       <c r="U174" s="4"/>
       <c r="Z174" s="9"/>
@@ -3441,7 +3264,6 @@
       <c r="L175" s="20"/>
       <c r="M175" s="22"/>
       <c r="N175" s="4"/>
-      <c r="O175" s="30"/>
       <c r="T175" s="9"/>
       <c r="U175" s="4"/>
       <c r="Z175" s="9"/>
@@ -3452,7 +3274,6 @@
       <c r="L176" s="20"/>
       <c r="M176" s="22"/>
       <c r="N176" s="4"/>
-      <c r="O176" s="30"/>
       <c r="T176" s="9"/>
       <c r="U176" s="4"/>
       <c r="Z176" s="9"/>
@@ -3463,7 +3284,6 @@
       <c r="L177" s="20"/>
       <c r="M177" s="22"/>
       <c r="N177" s="4"/>
-      <c r="O177" s="30"/>
       <c r="T177" s="9"/>
       <c r="U177" s="4"/>
       <c r="Z177" s="9"/>
@@ -3474,7 +3294,6 @@
       <c r="L178" s="20"/>
       <c r="M178" s="22"/>
       <c r="N178" s="4"/>
-      <c r="O178" s="30"/>
       <c r="T178" s="9"/>
       <c r="U178" s="4"/>
       <c r="Z178" s="9"/>
@@ -3485,7 +3304,6 @@
       <c r="L179" s="20"/>
       <c r="M179" s="22"/>
       <c r="N179" s="4"/>
-      <c r="O179" s="30"/>
       <c r="T179" s="9"/>
       <c r="U179" s="4"/>
       <c r="Z179" s="9"/>
@@ -3496,7 +3314,6 @@
       <c r="L180" s="20"/>
       <c r="M180" s="22"/>
       <c r="N180" s="4"/>
-      <c r="O180" s="30"/>
       <c r="T180" s="9"/>
       <c r="U180" s="4"/>
       <c r="Z180" s="9"/>
@@ -3507,7 +3324,6 @@
       <c r="L181" s="20"/>
       <c r="M181" s="22"/>
       <c r="N181" s="4"/>
-      <c r="O181" s="30"/>
       <c r="T181" s="9"/>
       <c r="U181" s="4"/>
       <c r="Z181" s="9"/>
@@ -3518,7 +3334,6 @@
       <c r="L182" s="20"/>
       <c r="M182" s="22"/>
       <c r="N182" s="4"/>
-      <c r="O182" s="30"/>
       <c r="T182" s="9"/>
       <c r="U182" s="4"/>
       <c r="Z182" s="9"/>
@@ -3529,7 +3344,6 @@
       <c r="L183" s="20"/>
       <c r="M183" s="22"/>
       <c r="N183" s="4"/>
-      <c r="O183" s="30"/>
       <c r="T183" s="9"/>
       <c r="U183" s="4"/>
       <c r="Z183" s="9"/>
@@ -3540,7 +3354,6 @@
       <c r="L184" s="20"/>
       <c r="M184" s="22"/>
       <c r="N184" s="4"/>
-      <c r="O184" s="30"/>
       <c r="T184" s="9"/>
       <c r="U184" s="4"/>
       <c r="Z184" s="9"/>
@@ -3551,7 +3364,6 @@
       <c r="L185" s="20"/>
       <c r="M185" s="22"/>
       <c r="N185" s="4"/>
-      <c r="O185" s="30"/>
       <c r="T185" s="9"/>
       <c r="U185" s="4"/>
       <c r="Z185" s="9"/>
@@ -3562,7 +3374,6 @@
       <c r="L186" s="20"/>
       <c r="M186" s="22"/>
       <c r="N186" s="4"/>
-      <c r="O186" s="30"/>
       <c r="T186" s="9"/>
       <c r="U186" s="4"/>
       <c r="Z186" s="9"/>
@@ -3573,7 +3384,6 @@
       <c r="L187" s="20"/>
       <c r="M187" s="22"/>
       <c r="N187" s="4"/>
-      <c r="O187" s="30"/>
       <c r="T187" s="9"/>
       <c r="U187" s="4"/>
       <c r="Z187" s="9"/>
@@ -3584,7 +3394,6 @@
       <c r="L188" s="20"/>
       <c r="M188" s="22"/>
       <c r="N188" s="4"/>
-      <c r="O188" s="30"/>
       <c r="T188" s="9"/>
       <c r="U188" s="4"/>
       <c r="Z188" s="9"/>
@@ -3595,7 +3404,6 @@
       <c r="L189" s="20"/>
       <c r="M189" s="22"/>
       <c r="N189" s="4"/>
-      <c r="O189" s="30"/>
       <c r="T189" s="9"/>
       <c r="U189" s="4"/>
       <c r="Z189" s="9"/>
@@ -3606,7 +3414,6 @@
       <c r="L190" s="20"/>
       <c r="M190" s="22"/>
       <c r="N190" s="4"/>
-      <c r="O190" s="30"/>
       <c r="T190" s="9"/>
       <c r="U190" s="4"/>
       <c r="Z190" s="9"/>
@@ -3617,7 +3424,6 @@
       <c r="L191" s="20"/>
       <c r="M191" s="22"/>
       <c r="N191" s="4"/>
-      <c r="O191" s="30"/>
       <c r="T191" s="9"/>
       <c r="U191" s="4"/>
       <c r="Z191" s="9"/>
@@ -3628,7 +3434,6 @@
       <c r="L192" s="20"/>
       <c r="M192" s="22"/>
       <c r="N192" s="4"/>
-      <c r="O192" s="30"/>
       <c r="T192" s="9"/>
       <c r="U192" s="4"/>
       <c r="Z192" s="9"/>
@@ -3639,7 +3444,6 @@
       <c r="L193" s="20"/>
       <c r="M193" s="22"/>
       <c r="N193" s="4"/>
-      <c r="O193" s="30"/>
       <c r="T193" s="9"/>
       <c r="U193" s="4"/>
       <c r="Z193" s="9"/>
@@ -3650,7 +3454,6 @@
       <c r="L194" s="20"/>
       <c r="M194" s="22"/>
       <c r="N194" s="4"/>
-      <c r="O194" s="30"/>
       <c r="T194" s="9"/>
       <c r="U194" s="4"/>
       <c r="Z194" s="9"/>
@@ -3661,7 +3464,6 @@
       <c r="L195" s="20"/>
       <c r="M195" s="22"/>
       <c r="N195" s="4"/>
-      <c r="O195" s="30"/>
       <c r="T195" s="9"/>
       <c r="U195" s="4"/>
       <c r="Z195" s="9"/>
@@ -3672,7 +3474,6 @@
       <c r="L196" s="20"/>
       <c r="M196" s="22"/>
       <c r="N196" s="4"/>
-      <c r="O196" s="30"/>
       <c r="T196" s="9"/>
       <c r="U196" s="4"/>
       <c r="Z196" s="9"/>
@@ -3683,7 +3484,6 @@
       <c r="L197" s="20"/>
       <c r="M197" s="22"/>
       <c r="N197" s="4"/>
-      <c r="O197" s="30"/>
       <c r="T197" s="9"/>
       <c r="U197" s="4"/>
       <c r="Z197" s="9"/>
@@ -3694,7 +3494,6 @@
       <c r="L198" s="20"/>
       <c r="M198" s="22"/>
       <c r="N198" s="4"/>
-      <c r="O198" s="30"/>
       <c r="T198" s="9"/>
       <c r="U198" s="4"/>
       <c r="Z198" s="9"/>
@@ -3705,7 +3504,6 @@
       <c r="L199" s="20"/>
       <c r="M199" s="22"/>
       <c r="N199" s="4"/>
-      <c r="O199" s="30"/>
       <c r="T199" s="9"/>
       <c r="U199" s="4"/>
       <c r="Z199" s="9"/>
@@ -3716,7 +3514,6 @@
       <c r="L200" s="20"/>
       <c r="M200" s="22"/>
       <c r="N200" s="4"/>
-      <c r="O200" s="30"/>
       <c r="T200" s="9"/>
       <c r="U200" s="4"/>
       <c r="Z200" s="9"/>
@@ -3727,7 +3524,6 @@
       <c r="L201" s="20"/>
       <c r="M201" s="22"/>
       <c r="N201" s="4"/>
-      <c r="O201" s="30"/>
       <c r="T201" s="9"/>
       <c r="U201" s="4"/>
       <c r="Z201" s="9"/>
@@ -3738,7 +3534,6 @@
       <c r="L202" s="20"/>
       <c r="M202" s="22"/>
       <c r="N202" s="4"/>
-      <c r="O202" s="30"/>
       <c r="T202" s="9"/>
       <c r="U202" s="4"/>
       <c r="Z202" s="9"/>
@@ -3749,7 +3544,6 @@
       <c r="L203" s="20"/>
       <c r="M203" s="22"/>
       <c r="N203" s="4"/>
-      <c r="O203" s="30"/>
       <c r="T203" s="9"/>
       <c r="U203" s="4"/>
       <c r="Z203" s="9"/>
@@ -3760,7 +3554,6 @@
       <c r="L204" s="20"/>
       <c r="M204" s="22"/>
       <c r="N204" s="4"/>
-      <c r="O204" s="30"/>
       <c r="T204" s="9"/>
       <c r="U204" s="4"/>
       <c r="Z204" s="9"/>
@@ -3771,7 +3564,6 @@
       <c r="L205" s="20"/>
       <c r="M205" s="22"/>
       <c r="N205" s="4"/>
-      <c r="O205" s="30"/>
       <c r="T205" s="9"/>
       <c r="U205" s="4"/>
       <c r="Z205" s="9"/>
@@ -3782,7 +3574,6 @@
       <c r="L206" s="20"/>
       <c r="M206" s="22"/>
       <c r="N206" s="4"/>
-      <c r="O206" s="30"/>
       <c r="T206" s="9"/>
       <c r="U206" s="4"/>
       <c r="Z206" s="9"/>
@@ -3793,7 +3584,6 @@
       <c r="L207" s="20"/>
       <c r="M207" s="22"/>
       <c r="N207" s="4"/>
-      <c r="O207" s="30"/>
       <c r="T207" s="9"/>
       <c r="U207" s="4"/>
       <c r="Z207" s="9"/>
@@ -3804,7 +3594,6 @@
       <c r="L208" s="20"/>
       <c r="M208" s="22"/>
       <c r="N208" s="4"/>
-      <c r="O208" s="30"/>
       <c r="T208" s="9"/>
       <c r="U208" s="4"/>
       <c r="Z208" s="9"/>
@@ -3815,7 +3604,6 @@
       <c r="L209" s="20"/>
       <c r="M209" s="22"/>
       <c r="N209" s="4"/>
-      <c r="O209" s="30"/>
       <c r="T209" s="9"/>
       <c r="U209" s="4"/>
       <c r="Z209" s="9"/>
@@ -3826,7 +3614,6 @@
       <c r="L210" s="20"/>
       <c r="M210" s="22"/>
       <c r="N210" s="4"/>
-      <c r="O210" s="30"/>
       <c r="T210" s="9"/>
       <c r="U210" s="4"/>
       <c r="Z210" s="9"/>
@@ -3837,7 +3624,6 @@
       <c r="L211" s="20"/>
       <c r="M211" s="22"/>
       <c r="N211" s="4"/>
-      <c r="O211" s="30"/>
       <c r="T211" s="9"/>
       <c r="U211" s="4"/>
       <c r="Z211" s="9"/>
@@ -3848,7 +3634,6 @@
       <c r="L212" s="20"/>
       <c r="M212" s="22"/>
       <c r="N212" s="4"/>
-      <c r="O212" s="30"/>
       <c r="T212" s="9"/>
       <c r="U212" s="4"/>
       <c r="Z212" s="9"/>
@@ -3859,7 +3644,6 @@
       <c r="L213" s="20"/>
       <c r="M213" s="22"/>
       <c r="N213" s="4"/>
-      <c r="O213" s="30"/>
       <c r="T213" s="9"/>
       <c r="U213" s="4"/>
       <c r="Z213" s="9"/>
@@ -3870,7 +3654,6 @@
       <c r="L214" s="20"/>
       <c r="M214" s="22"/>
       <c r="N214" s="4"/>
-      <c r="O214" s="30"/>
       <c r="T214" s="9"/>
       <c r="U214" s="4"/>
       <c r="Z214" s="9"/>
@@ -3881,7 +3664,6 @@
       <c r="L215" s="20"/>
       <c r="M215" s="22"/>
       <c r="N215" s="4"/>
-      <c r="O215" s="30"/>
       <c r="T215" s="9"/>
       <c r="U215" s="4"/>
       <c r="Z215" s="9"/>
@@ -3892,7 +3674,6 @@
       <c r="L216" s="20"/>
       <c r="M216" s="22"/>
       <c r="N216" s="4"/>
-      <c r="O216" s="30"/>
       <c r="T216" s="9"/>
       <c r="U216" s="4"/>
       <c r="Z216" s="9"/>
@@ -3903,7 +3684,6 @@
       <c r="L217" s="20"/>
       <c r="M217" s="22"/>
       <c r="N217" s="4"/>
-      <c r="O217" s="30"/>
       <c r="T217" s="9"/>
       <c r="U217" s="4"/>
       <c r="Z217" s="9"/>
@@ -3914,7 +3694,6 @@
       <c r="L218" s="20"/>
       <c r="M218" s="22"/>
       <c r="N218" s="4"/>
-      <c r="O218" s="30"/>
       <c r="T218" s="9"/>
       <c r="U218" s="4"/>
       <c r="Z218" s="9"/>
@@ -3925,7 +3704,6 @@
       <c r="L219" s="20"/>
       <c r="M219" s="22"/>
       <c r="N219" s="4"/>
-      <c r="O219" s="30"/>
       <c r="T219" s="9"/>
       <c r="U219" s="4"/>
       <c r="Z219" s="9"/>
@@ -3936,7 +3714,6 @@
       <c r="L220" s="20"/>
       <c r="M220" s="22"/>
       <c r="N220" s="4"/>
-      <c r="O220" s="30"/>
       <c r="T220" s="9"/>
       <c r="U220" s="4"/>
       <c r="Z220" s="9"/>
@@ -3947,7 +3724,6 @@
       <c r="L221" s="20"/>
       <c r="M221" s="22"/>
       <c r="N221" s="4"/>
-      <c r="O221" s="30"/>
       <c r="T221" s="9"/>
       <c r="U221" s="4"/>
       <c r="Z221" s="9"/>
@@ -3958,7 +3734,6 @@
       <c r="L222" s="20"/>
       <c r="M222" s="22"/>
       <c r="N222" s="4"/>
-      <c r="O222" s="30"/>
       <c r="T222" s="9"/>
       <c r="U222" s="4"/>
       <c r="Z222" s="9"/>
@@ -3969,7 +3744,6 @@
       <c r="L223" s="20"/>
       <c r="M223" s="22"/>
       <c r="N223" s="4"/>
-      <c r="O223" s="30"/>
       <c r="T223" s="9"/>
       <c r="U223" s="4"/>
       <c r="Z223" s="9"/>
@@ -3980,7 +3754,6 @@
       <c r="L224" s="20"/>
       <c r="M224" s="22"/>
       <c r="N224" s="4"/>
-      <c r="O224" s="30"/>
       <c r="T224" s="9"/>
       <c r="U224" s="4"/>
       <c r="Z224" s="9"/>
@@ -3991,7 +3764,6 @@
       <c r="L225" s="20"/>
       <c r="M225" s="22"/>
       <c r="N225" s="4"/>
-      <c r="O225" s="30"/>
       <c r="T225" s="9"/>
       <c r="U225" s="4"/>
       <c r="Z225" s="9"/>
@@ -4002,7 +3774,6 @@
       <c r="L226" s="20"/>
       <c r="M226" s="22"/>
       <c r="N226" s="4"/>
-      <c r="O226" s="30"/>
       <c r="T226" s="9"/>
       <c r="U226" s="4"/>
       <c r="Z226" s="9"/>
@@ -4013,7 +3784,6 @@
       <c r="L227" s="20"/>
       <c r="M227" s="22"/>
       <c r="N227" s="4"/>
-      <c r="O227" s="30"/>
       <c r="T227" s="9"/>
       <c r="U227" s="4"/>
       <c r="Z227" s="9"/>
@@ -4024,7 +3794,6 @@
       <c r="L228" s="20"/>
       <c r="M228" s="22"/>
       <c r="N228" s="4"/>
-      <c r="O228" s="30"/>
       <c r="T228" s="9"/>
       <c r="U228" s="4"/>
       <c r="Z228" s="9"/>
@@ -4035,7 +3804,6 @@
       <c r="L229" s="20"/>
       <c r="M229" s="22"/>
       <c r="N229" s="4"/>
-      <c r="O229" s="30"/>
       <c r="T229" s="9"/>
       <c r="U229" s="4"/>
       <c r="Z229" s="9"/>
@@ -4046,7 +3814,6 @@
       <c r="L230" s="20"/>
       <c r="M230" s="22"/>
       <c r="N230" s="4"/>
-      <c r="O230" s="30"/>
       <c r="T230" s="9"/>
       <c r="U230" s="4"/>
       <c r="Z230" s="9"/>
@@ -4057,7 +3824,6 @@
       <c r="L231" s="20"/>
       <c r="M231" s="22"/>
       <c r="N231" s="4"/>
-      <c r="O231" s="30"/>
       <c r="T231" s="9"/>
       <c r="U231" s="4"/>
       <c r="Z231" s="9"/>
@@ -4068,7 +3834,6 @@
       <c r="L232" s="20"/>
       <c r="M232" s="22"/>
       <c r="N232" s="4"/>
-      <c r="O232" s="30"/>
       <c r="T232" s="9"/>
       <c r="U232" s="4"/>
       <c r="Z232" s="9"/>
@@ -4079,7 +3844,6 @@
       <c r="L233" s="20"/>
       <c r="M233" s="22"/>
       <c r="N233" s="4"/>
-      <c r="O233" s="30"/>
       <c r="T233" s="9"/>
       <c r="U233" s="4"/>
       <c r="Z233" s="9"/>
@@ -4090,7 +3854,6 @@
       <c r="L234" s="20"/>
       <c r="M234" s="22"/>
       <c r="N234" s="4"/>
-      <c r="O234" s="30"/>
       <c r="T234" s="9"/>
       <c r="U234" s="4"/>
       <c r="Z234" s="9"/>
@@ -4101,7 +3864,6 @@
       <c r="L235" s="20"/>
       <c r="M235" s="22"/>
       <c r="N235" s="4"/>
-      <c r="O235" s="30"/>
       <c r="T235" s="9"/>
       <c r="U235" s="4"/>
       <c r="Z235" s="9"/>
@@ -4112,7 +3874,6 @@
       <c r="L236" s="20"/>
       <c r="M236" s="22"/>
       <c r="N236" s="4"/>
-      <c r="O236" s="30"/>
       <c r="T236" s="9"/>
       <c r="U236" s="4"/>
       <c r="Z236" s="9"/>
@@ -4123,7 +3884,6 @@
       <c r="L237" s="20"/>
       <c r="M237" s="22"/>
       <c r="N237" s="4"/>
-      <c r="O237" s="30"/>
       <c r="T237" s="9"/>
       <c r="U237" s="4"/>
       <c r="Z237" s="9"/>
@@ -4134,7 +3894,6 @@
       <c r="L238" s="20"/>
       <c r="M238" s="22"/>
       <c r="N238" s="4"/>
-      <c r="O238" s="30"/>
       <c r="T238" s="9"/>
       <c r="U238" s="4"/>
       <c r="Z238" s="9"/>
@@ -4145,7 +3904,6 @@
       <c r="L239" s="20"/>
       <c r="M239" s="22"/>
       <c r="N239" s="4"/>
-      <c r="O239" s="30"/>
       <c r="T239" s="9"/>
       <c r="U239" s="4"/>
       <c r="Z239" s="9"/>
@@ -4156,7 +3914,6 @@
       <c r="L240" s="20"/>
       <c r="M240" s="22"/>
       <c r="N240" s="4"/>
-      <c r="O240" s="30"/>
       <c r="T240" s="9"/>
       <c r="U240" s="4"/>
       <c r="Z240" s="9"/>
@@ -4167,7 +3924,6 @@
       <c r="L241" s="20"/>
       <c r="M241" s="22"/>
       <c r="N241" s="4"/>
-      <c r="O241" s="30"/>
       <c r="T241" s="9"/>
       <c r="U241" s="4"/>
       <c r="Z241" s="9"/>
@@ -4178,7 +3934,6 @@
       <c r="L242" s="20"/>
       <c r="M242" s="22"/>
       <c r="N242" s="4"/>
-      <c r="O242" s="30"/>
       <c r="T242" s="9"/>
       <c r="U242" s="4"/>
       <c r="Z242" s="9"/>
@@ -4189,7 +3944,6 @@
       <c r="L243" s="20"/>
       <c r="M243" s="22"/>
       <c r="N243" s="4"/>
-      <c r="O243" s="30"/>
       <c r="T243" s="9"/>
       <c r="U243" s="4"/>
       <c r="Z243" s="9"/>
@@ -4200,7 +3954,6 @@
       <c r="L244" s="20"/>
       <c r="M244" s="22"/>
       <c r="N244" s="4"/>
-      <c r="O244" s="30"/>
       <c r="T244" s="9"/>
       <c r="U244" s="4"/>
       <c r="Z244" s="9"/>
@@ -4211,7 +3964,6 @@
       <c r="L245" s="20"/>
       <c r="M245" s="22"/>
       <c r="N245" s="4"/>
-      <c r="O245" s="30"/>
       <c r="T245" s="9"/>
       <c r="U245" s="4"/>
       <c r="Z245" s="9"/>
@@ -4222,7 +3974,6 @@
       <c r="L246" s="20"/>
       <c r="M246" s="22"/>
       <c r="N246" s="4"/>
-      <c r="O246" s="30"/>
       <c r="T246" s="9"/>
       <c r="U246" s="4"/>
       <c r="Z246" s="9"/>
@@ -4233,7 +3984,6 @@
       <c r="L247" s="20"/>
       <c r="M247" s="22"/>
       <c r="N247" s="4"/>
-      <c r="O247" s="30"/>
       <c r="T247" s="9"/>
       <c r="U247" s="4"/>
       <c r="Z247" s="9"/>
@@ -4244,7 +3994,6 @@
       <c r="L248" s="20"/>
       <c r="M248" s="22"/>
       <c r="N248" s="4"/>
-      <c r="O248" s="30"/>
       <c r="T248" s="9"/>
       <c r="U248" s="4"/>
       <c r="Z248" s="9"/>
@@ -4255,7 +4004,6 @@
       <c r="L249" s="20"/>
       <c r="M249" s="22"/>
       <c r="N249" s="4"/>
-      <c r="O249" s="30"/>
       <c r="T249" s="9"/>
       <c r="U249" s="4"/>
       <c r="Z249" s="9"/>
@@ -4266,7 +4014,6 @@
       <c r="L250" s="20"/>
       <c r="M250" s="22"/>
       <c r="N250" s="4"/>
-      <c r="O250" s="30"/>
       <c r="T250" s="9"/>
       <c r="U250" s="4"/>
       <c r="Z250" s="9"/>
@@ -4277,7 +4024,6 @@
       <c r="L251" s="20"/>
       <c r="M251" s="22"/>
       <c r="N251" s="4"/>
-      <c r="O251" s="30"/>
       <c r="T251" s="9"/>
       <c r="U251" s="4"/>
       <c r="Z251" s="9"/>
@@ -4288,7 +4034,6 @@
       <c r="L252" s="20"/>
       <c r="M252" s="22"/>
       <c r="N252" s="4"/>
-      <c r="O252" s="30"/>
       <c r="T252" s="9"/>
       <c r="U252" s="4"/>
       <c r="Z252" s="9"/>
@@ -4299,7 +4044,6 @@
       <c r="L253" s="20"/>
       <c r="M253" s="22"/>
       <c r="N253" s="4"/>
-      <c r="O253" s="30"/>
       <c r="T253" s="9"/>
       <c r="U253" s="4"/>
       <c r="Z253" s="9"/>
@@ -4310,7 +4054,6 @@
       <c r="L254" s="20"/>
       <c r="M254" s="22"/>
       <c r="N254" s="4"/>
-      <c r="O254" s="30"/>
       <c r="T254" s="9"/>
       <c r="U254" s="4"/>
       <c r="Z254" s="9"/>
@@ -4321,7 +4064,6 @@
       <c r="L255" s="20"/>
       <c r="M255" s="22"/>
       <c r="N255" s="4"/>
-      <c r="O255" s="30"/>
       <c r="T255" s="9"/>
       <c r="U255" s="4"/>
       <c r="Z255" s="9"/>
@@ -4332,7 +4074,6 @@
       <c r="L256" s="20"/>
       <c r="M256" s="22"/>
       <c r="N256" s="4"/>
-      <c r="O256" s="30"/>
       <c r="T256" s="9"/>
       <c r="U256" s="4"/>
       <c r="Z256" s="9"/>
@@ -4343,7 +4084,6 @@
       <c r="L257" s="20"/>
       <c r="M257" s="22"/>
       <c r="N257" s="4"/>
-      <c r="O257" s="30"/>
       <c r="T257" s="9"/>
       <c r="U257" s="4"/>
       <c r="Z257" s="9"/>
@@ -4354,7 +4094,6 @@
       <c r="L258" s="20"/>
       <c r="M258" s="22"/>
       <c r="N258" s="4"/>
-      <c r="O258" s="30"/>
       <c r="T258" s="9"/>
       <c r="U258" s="4"/>
       <c r="Z258" s="9"/>
@@ -4365,7 +4104,6 @@
       <c r="L259" s="20"/>
       <c r="M259" s="22"/>
       <c r="N259" s="4"/>
-      <c r="O259" s="30"/>
       <c r="T259" s="9"/>
       <c r="U259" s="4"/>
       <c r="Z259" s="9"/>
@@ -4376,7 +4114,6 @@
       <c r="L260" s="20"/>
       <c r="M260" s="22"/>
       <c r="N260" s="4"/>
-      <c r="O260" s="30"/>
       <c r="T260" s="9"/>
       <c r="U260" s="4"/>
       <c r="Z260" s="9"/>
@@ -4387,7 +4124,6 @@
       <c r="L261" s="20"/>
       <c r="M261" s="22"/>
       <c r="N261" s="4"/>
-      <c r="O261" s="30"/>
       <c r="T261" s="9"/>
       <c r="U261" s="4"/>
       <c r="Z261" s="9"/>
@@ -4398,7 +4134,6 @@
       <c r="L262" s="20"/>
       <c r="M262" s="22"/>
       <c r="N262" s="4"/>
-      <c r="O262" s="30"/>
       <c r="T262" s="9"/>
       <c r="U262" s="4"/>
       <c r="Z262" s="9"/>
@@ -4409,7 +4144,6 @@
       <c r="L263" s="20"/>
       <c r="M263" s="22"/>
       <c r="N263" s="4"/>
-      <c r="O263" s="30"/>
       <c r="T263" s="9"/>
       <c r="U263" s="4"/>
       <c r="Z263" s="9"/>
@@ -4420,7 +4154,6 @@
       <c r="L264" s="20"/>
       <c r="M264" s="22"/>
       <c r="N264" s="4"/>
-      <c r="O264" s="30"/>
       <c r="T264" s="9"/>
       <c r="U264" s="4"/>
       <c r="Z264" s="9"/>
@@ -4431,7 +4164,6 @@
       <c r="L265" s="20"/>
       <c r="M265" s="22"/>
       <c r="N265" s="4"/>
-      <c r="O265" s="30"/>
       <c r="T265" s="9"/>
       <c r="U265" s="4"/>
       <c r="Z265" s="9"/>
@@ -4442,7 +4174,6 @@
       <c r="L266" s="20"/>
       <c r="M266" s="22"/>
       <c r="N266" s="4"/>
-      <c r="O266" s="30"/>
       <c r="T266" s="9"/>
       <c r="U266" s="4"/>
       <c r="Z266" s="9"/>
@@ -4453,7 +4184,6 @@
       <c r="L267" s="20"/>
       <c r="M267" s="22"/>
       <c r="N267" s="4"/>
-      <c r="O267" s="30"/>
       <c r="T267" s="9"/>
       <c r="U267" s="4"/>
       <c r="Z267" s="9"/>
@@ -4464,7 +4194,6 @@
       <c r="L268" s="20"/>
       <c r="M268" s="22"/>
       <c r="N268" s="4"/>
-      <c r="O268" s="30"/>
       <c r="T268" s="9"/>
       <c r="U268" s="4"/>
       <c r="Z268" s="9"/>
@@ -4475,7 +4204,6 @@
       <c r="L269" s="20"/>
       <c r="M269" s="22"/>
       <c r="N269" s="4"/>
-      <c r="O269" s="30"/>
       <c r="T269" s="9"/>
       <c r="U269" s="4"/>
       <c r="Z269" s="9"/>
@@ -4486,7 +4214,6 @@
       <c r="L270" s="20"/>
       <c r="M270" s="22"/>
       <c r="N270" s="4"/>
-      <c r="O270" s="30"/>
       <c r="T270" s="9"/>
       <c r="U270" s="4"/>
       <c r="Z270" s="9"/>
@@ -4497,7 +4224,6 @@
       <c r="L271" s="20"/>
       <c r="M271" s="22"/>
       <c r="N271" s="4"/>
-      <c r="O271" s="30"/>
       <c r="T271" s="9"/>
       <c r="U271" s="4"/>
       <c r="Z271" s="9"/>
@@ -4508,7 +4234,6 @@
       <c r="L272" s="20"/>
       <c r="M272" s="22"/>
       <c r="N272" s="4"/>
-      <c r="O272" s="30"/>
       <c r="T272" s="9"/>
       <c r="U272" s="4"/>
       <c r="Z272" s="9"/>
@@ -4519,7 +4244,6 @@
       <c r="L273" s="20"/>
       <c r="M273" s="22"/>
       <c r="N273" s="4"/>
-      <c r="O273" s="30"/>
       <c r="T273" s="9"/>
       <c r="U273" s="4"/>
       <c r="Z273" s="9"/>
@@ -4530,7 +4254,6 @@
       <c r="L274" s="20"/>
       <c r="M274" s="22"/>
       <c r="N274" s="4"/>
-      <c r="O274" s="30"/>
       <c r="T274" s="9"/>
       <c r="U274" s="4"/>
       <c r="Z274" s="9"/>
@@ -4541,7 +4264,6 @@
       <c r="L275" s="20"/>
       <c r="M275" s="22"/>
       <c r="N275" s="4"/>
-      <c r="O275" s="30"/>
       <c r="T275" s="9"/>
       <c r="U275" s="4"/>
       <c r="Z275" s="9"/>
@@ -4552,7 +4274,6 @@
       <c r="L276" s="20"/>
       <c r="M276" s="22"/>
       <c r="N276" s="4"/>
-      <c r="O276" s="30"/>
       <c r="T276" s="9"/>
       <c r="U276" s="4"/>
       <c r="Z276" s="9"/>
@@ -4563,7 +4284,6 @@
       <c r="L277" s="20"/>
       <c r="M277" s="22"/>
       <c r="N277" s="4"/>
-      <c r="O277" s="30"/>
       <c r="T277" s="9"/>
       <c r="U277" s="4"/>
       <c r="Z277" s="9"/>
@@ -4574,7 +4294,6 @@
       <c r="L278" s="20"/>
       <c r="M278" s="22"/>
       <c r="N278" s="4"/>
-      <c r="O278" s="30"/>
       <c r="T278" s="9"/>
       <c r="U278" s="4"/>
       <c r="Z278" s="9"/>
@@ -4585,7 +4304,6 @@
       <c r="L279" s="20"/>
       <c r="M279" s="22"/>
       <c r="N279" s="4"/>
-      <c r="O279" s="30"/>
       <c r="T279" s="9"/>
       <c r="U279" s="4"/>
       <c r="Z279" s="9"/>
@@ -4596,7 +4314,6 @@
       <c r="L280" s="20"/>
       <c r="M280" s="22"/>
       <c r="N280" s="4"/>
-      <c r="O280" s="30"/>
       <c r="T280" s="9"/>
       <c r="U280" s="4"/>
       <c r="Z280" s="9"/>
@@ -4607,7 +4324,6 @@
       <c r="L281" s="20"/>
       <c r="M281" s="22"/>
       <c r="N281" s="4"/>
-      <c r="O281" s="30"/>
       <c r="T281" s="9"/>
       <c r="U281" s="4"/>
       <c r="Z281" s="9"/>
@@ -4618,7 +4334,6 @@
       <c r="L282" s="20"/>
       <c r="M282" s="22"/>
       <c r="N282" s="4"/>
-      <c r="O282" s="30"/>
       <c r="T282" s="9"/>
       <c r="U282" s="4"/>
       <c r="Z282" s="9"/>
@@ -4629,7 +4344,6 @@
       <c r="L283" s="20"/>
       <c r="M283" s="22"/>
       <c r="N283" s="4"/>
-      <c r="O283" s="30"/>
       <c r="T283" s="9"/>
       <c r="U283" s="4"/>
       <c r="Z283" s="9"/>
@@ -4640,7 +4354,6 @@
       <c r="L284" s="20"/>
       <c r="M284" s="22"/>
       <c r="N284" s="4"/>
-      <c r="O284" s="30"/>
       <c r="T284" s="9"/>
       <c r="U284" s="4"/>
       <c r="Z284" s="9"/>
@@ -4651,7 +4364,6 @@
       <c r="L285" s="20"/>
       <c r="M285" s="22"/>
       <c r="N285" s="4"/>
-      <c r="O285" s="30"/>
       <c r="T285" s="9"/>
       <c r="U285" s="4"/>
       <c r="Z285" s="9"/>
@@ -4662,7 +4374,6 @@
       <c r="L286" s="20"/>
       <c r="M286" s="22"/>
       <c r="N286" s="4"/>
-      <c r="O286" s="30"/>
       <c r="T286" s="9"/>
       <c r="U286" s="4"/>
       <c r="Z286" s="9"/>
@@ -4673,7 +4384,6 @@
       <c r="L287" s="20"/>
       <c r="M287" s="22"/>
       <c r="N287" s="4"/>
-      <c r="O287" s="30"/>
       <c r="T287" s="9"/>
       <c r="U287" s="4"/>
       <c r="Z287" s="9"/>
@@ -4684,7 +4394,6 @@
       <c r="L288" s="20"/>
       <c r="M288" s="22"/>
       <c r="N288" s="4"/>
-      <c r="O288" s="30"/>
       <c r="T288" s="9"/>
       <c r="U288" s="4"/>
       <c r="Z288" s="9"/>
@@ -4695,7 +4404,6 @@
       <c r="L289" s="20"/>
       <c r="M289" s="22"/>
       <c r="N289" s="4"/>
-      <c r="O289" s="30"/>
       <c r="T289" s="9"/>
       <c r="U289" s="4"/>
       <c r="Z289" s="9"/>
@@ -4706,7 +4414,6 @@
       <c r="L290" s="20"/>
       <c r="M290" s="22"/>
       <c r="N290" s="4"/>
-      <c r="O290" s="30"/>
       <c r="T290" s="9"/>
       <c r="U290" s="4"/>
       <c r="Z290" s="9"/>
@@ -4717,7 +4424,6 @@
       <c r="L291" s="20"/>
       <c r="M291" s="22"/>
       <c r="N291" s="4"/>
-      <c r="O291" s="30"/>
       <c r="T291" s="9"/>
       <c r="U291" s="4"/>
       <c r="Z291" s="9"/>
@@ -4728,7 +4434,6 @@
       <c r="L292" s="20"/>
       <c r="M292" s="22"/>
       <c r="N292" s="4"/>
-      <c r="O292" s="30"/>
       <c r="T292" s="9"/>
       <c r="U292" s="4"/>
       <c r="Z292" s="9"/>
@@ -4739,7 +4444,6 @@
       <c r="L293" s="20"/>
       <c r="M293" s="22"/>
       <c r="N293" s="4"/>
-      <c r="O293" s="30"/>
       <c r="T293" s="9"/>
       <c r="U293" s="4"/>
       <c r="Z293" s="9"/>
@@ -4750,7 +4454,6 @@
       <c r="L294" s="20"/>
       <c r="M294" s="22"/>
       <c r="N294" s="4"/>
-      <c r="O294" s="30"/>
       <c r="T294" s="9"/>
       <c r="U294" s="4"/>
       <c r="Z294" s="9"/>
@@ -4761,7 +4464,6 @@
       <c r="L295" s="20"/>
       <c r="M295" s="22"/>
       <c r="N295" s="4"/>
-      <c r="O295" s="30"/>
       <c r="T295" s="9"/>
       <c r="U295" s="4"/>
       <c r="Z295" s="9"/>
@@ -4772,7 +4474,6 @@
       <c r="L296" s="20"/>
       <c r="M296" s="22"/>
       <c r="N296" s="4"/>
-      <c r="O296" s="30"/>
       <c r="T296" s="9"/>
       <c r="U296" s="4"/>
       <c r="Z296" s="9"/>
@@ -4783,7 +4484,6 @@
       <c r="L297" s="20"/>
       <c r="M297" s="22"/>
       <c r="N297" s="4"/>
-      <c r="O297" s="30"/>
       <c r="T297" s="9"/>
       <c r="U297" s="4"/>
       <c r="Z297" s="9"/>
@@ -4794,7 +4494,6 @@
       <c r="L298" s="20"/>
       <c r="M298" s="22"/>
       <c r="N298" s="4"/>
-      <c r="O298" s="30"/>
       <c r="T298" s="9"/>
       <c r="U298" s="4"/>
       <c r="Z298" s="9"/>
@@ -4805,7 +4504,6 @@
       <c r="L299" s="20"/>
       <c r="M299" s="22"/>
       <c r="N299" s="4"/>
-      <c r="O299" s="30"/>
       <c r="T299" s="9"/>
       <c r="U299" s="4"/>
       <c r="Z299" s="9"/>
@@ -4816,7 +4514,6 @@
       <c r="L300" s="20"/>
       <c r="M300" s="22"/>
       <c r="N300" s="4"/>
-      <c r="O300" s="30"/>
       <c r="T300" s="9"/>
       <c r="U300" s="4"/>
       <c r="Z300" s="9"/>
@@ -4827,7 +4524,6 @@
       <c r="L301" s="20"/>
       <c r="M301" s="22"/>
       <c r="N301" s="4"/>
-      <c r="O301" s="30"/>
       <c r="T301" s="9"/>
       <c r="U301" s="4"/>
       <c r="Z301" s="9"/>
@@ -4838,7 +4534,6 @@
       <c r="L302" s="20"/>
       <c r="M302" s="22"/>
       <c r="N302" s="4"/>
-      <c r="O302" s="30"/>
       <c r="T302" s="9"/>
       <c r="U302" s="4"/>
       <c r="Z302" s="9"/>
@@ -4849,7 +4544,6 @@
       <c r="L303" s="20"/>
       <c r="M303" s="22"/>
       <c r="N303" s="4"/>
-      <c r="O303" s="30"/>
       <c r="T303" s="9"/>
       <c r="U303" s="4"/>
       <c r="Z303" s="9"/>
@@ -4860,7 +4554,6 @@
       <c r="L304" s="20"/>
       <c r="M304" s="22"/>
       <c r="N304" s="4"/>
-      <c r="O304" s="30"/>
       <c r="T304" s="9"/>
       <c r="U304" s="4"/>
       <c r="Z304" s="9"/>
@@ -4871,7 +4564,6 @@
       <c r="L305" s="20"/>
       <c r="M305" s="22"/>
       <c r="N305" s="4"/>
-      <c r="O305" s="30"/>
       <c r="T305" s="9"/>
       <c r="U305" s="4"/>
       <c r="Z305" s="9"/>
@@ -4882,7 +4574,6 @@
       <c r="L306" s="20"/>
       <c r="M306" s="22"/>
       <c r="N306" s="4"/>
-      <c r="O306" s="30"/>
       <c r="T306" s="9"/>
       <c r="U306" s="4"/>
       <c r="Z306" s="9"/>
@@ -4893,7 +4584,6 @@
       <c r="L307" s="20"/>
       <c r="M307" s="22"/>
       <c r="N307" s="4"/>
-      <c r="O307" s="30"/>
       <c r="T307" s="9"/>
       <c r="U307" s="4"/>
       <c r="Z307" s="9"/>
@@ -4904,7 +4594,6 @@
       <c r="L308" s="20"/>
       <c r="M308" s="22"/>
       <c r="N308" s="4"/>
-      <c r="O308" s="30"/>
       <c r="T308" s="9"/>
       <c r="U308" s="4"/>
       <c r="Z308" s="9"/>
@@ -4915,7 +4604,6 @@
       <c r="L309" s="20"/>
       <c r="M309" s="22"/>
       <c r="N309" s="4"/>
-      <c r="O309" s="30"/>
       <c r="T309" s="9"/>
       <c r="U309" s="4"/>
       <c r="Z309" s="9"/>
@@ -4926,7 +4614,6 @@
       <c r="L310" s="20"/>
       <c r="M310" s="22"/>
       <c r="N310" s="4"/>
-      <c r="O310" s="30"/>
       <c r="T310" s="9"/>
       <c r="U310" s="4"/>
       <c r="Z310" s="9"/>
@@ -4937,7 +4624,6 @@
       <c r="L311" s="20"/>
       <c r="M311" s="22"/>
       <c r="N311" s="4"/>
-      <c r="O311" s="30"/>
       <c r="T311" s="9"/>
       <c r="U311" s="4"/>
       <c r="Z311" s="9"/>
@@ -4948,7 +4634,6 @@
       <c r="L312" s="20"/>
       <c r="M312" s="22"/>
       <c r="N312" s="4"/>
-      <c r="O312" s="30"/>
       <c r="T312" s="9"/>
       <c r="U312" s="4"/>
       <c r="Z312" s="9"/>
@@ -4959,7 +4644,6 @@
       <c r="L313" s="20"/>
       <c r="M313" s="22"/>
       <c r="N313" s="4"/>
-      <c r="O313" s="30"/>
       <c r="T313" s="9"/>
       <c r="U313" s="4"/>
       <c r="Z313" s="9"/>
@@ -4970,7 +4654,6 @@
       <c r="L314" s="20"/>
       <c r="M314" s="22"/>
       <c r="N314" s="4"/>
-      <c r="O314" s="30"/>
       <c r="T314" s="9"/>
       <c r="U314" s="4"/>
       <c r="Z314" s="9"/>
@@ -4981,7 +4664,6 @@
       <c r="L315" s="20"/>
       <c r="M315" s="22"/>
       <c r="N315" s="4"/>
-      <c r="O315" s="30"/>
       <c r="T315" s="9"/>
       <c r="U315" s="4"/>
       <c r="Z315" s="9"/>
@@ -4992,7 +4674,6 @@
       <c r="L316" s="20"/>
       <c r="M316" s="22"/>
       <c r="N316" s="4"/>
-      <c r="O316" s="30"/>
       <c r="T316" s="9"/>
       <c r="U316" s="4"/>
       <c r="Z316" s="9"/>
@@ -5003,7 +4684,6 @@
       <c r="L317" s="20"/>
       <c r="M317" s="22"/>
       <c r="N317" s="4"/>
-      <c r="O317" s="30"/>
       <c r="T317" s="9"/>
       <c r="U317" s="4"/>
       <c r="Z317" s="9"/>
@@ -5014,7 +4694,6 @@
       <c r="L318" s="20"/>
       <c r="M318" s="22"/>
       <c r="N318" s="4"/>
-      <c r="O318" s="30"/>
       <c r="T318" s="9"/>
       <c r="U318" s="4"/>
       <c r="Z318" s="9"/>
@@ -5025,7 +4704,6 @@
       <c r="L319" s="20"/>
       <c r="M319" s="22"/>
       <c r="N319" s="4"/>
-      <c r="O319" s="30"/>
       <c r="T319" s="9"/>
       <c r="U319" s="4"/>
       <c r="Z319" s="9"/>
@@ -5036,7 +4714,6 @@
       <c r="L320" s="20"/>
       <c r="M320" s="22"/>
       <c r="N320" s="4"/>
-      <c r="O320" s="30"/>
       <c r="T320" s="9"/>
       <c r="U320" s="4"/>
       <c r="Z320" s="9"/>
@@ -5047,7 +4724,6 @@
       <c r="L321" s="20"/>
       <c r="M321" s="22"/>
       <c r="N321" s="4"/>
-      <c r="O321" s="30"/>
       <c r="T321" s="9"/>
       <c r="U321" s="4"/>
       <c r="Z321" s="9"/>
@@ -5058,7 +4734,6 @@
       <c r="L322" s="20"/>
       <c r="M322" s="22"/>
       <c r="N322" s="4"/>
-      <c r="O322" s="30"/>
       <c r="T322" s="9"/>
       <c r="U322" s="4"/>
       <c r="Z322" s="9"/>
@@ -5069,7 +4744,6 @@
       <c r="L323" s="20"/>
       <c r="M323" s="22"/>
       <c r="N323" s="4"/>
-      <c r="O323" s="30"/>
       <c r="T323" s="9"/>
       <c r="U323" s="4"/>
       <c r="Z323" s="9"/>
@@ -5080,7 +4754,6 @@
       <c r="L324" s="20"/>
       <c r="M324" s="22"/>
       <c r="N324" s="4"/>
-      <c r="O324" s="30"/>
       <c r="T324" s="9"/>
       <c r="U324" s="4"/>
       <c r="Z324" s="9"/>
@@ -5091,7 +4764,6 @@
       <c r="L325" s="20"/>
       <c r="M325" s="22"/>
       <c r="N325" s="4"/>
-      <c r="O325" s="30"/>
       <c r="T325" s="9"/>
       <c r="U325" s="4"/>
       <c r="Z325" s="9"/>
@@ -5102,7 +4774,6 @@
       <c r="L326" s="20"/>
       <c r="M326" s="22"/>
       <c r="N326" s="4"/>
-      <c r="O326" s="30"/>
       <c r="T326" s="9"/>
       <c r="U326" s="4"/>
       <c r="Z326" s="9"/>
@@ -5113,7 +4784,6 @@
       <c r="L327" s="20"/>
       <c r="M327" s="22"/>
       <c r="N327" s="4"/>
-      <c r="O327" s="30"/>
       <c r="T327" s="9"/>
       <c r="U327" s="4"/>
       <c r="Z327" s="9"/>
@@ -5124,7 +4794,6 @@
       <c r="L328" s="20"/>
       <c r="M328" s="22"/>
       <c r="N328" s="4"/>
-      <c r="O328" s="30"/>
       <c r="T328" s="9"/>
       <c r="U328" s="4"/>
       <c r="Z328" s="9"/>
@@ -5135,7 +4804,6 @@
       <c r="L329" s="20"/>
       <c r="M329" s="22"/>
       <c r="N329" s="4"/>
-      <c r="O329" s="30"/>
       <c r="T329" s="9"/>
       <c r="U329" s="4"/>
       <c r="Z329" s="9"/>
@@ -5146,7 +4814,6 @@
       <c r="L330" s="20"/>
       <c r="M330" s="22"/>
       <c r="N330" s="4"/>
-      <c r="O330" s="30"/>
       <c r="T330" s="9"/>
       <c r="U330" s="4"/>
       <c r="Z330" s="9"/>
@@ -5157,7 +4824,6 @@
       <c r="L331" s="20"/>
       <c r="M331" s="22"/>
       <c r="N331" s="4"/>
-      <c r="O331" s="30"/>
       <c r="T331" s="9"/>
       <c r="U331" s="4"/>
       <c r="Z331" s="9"/>
@@ -5168,7 +4834,6 @@
       <c r="L332" s="20"/>
       <c r="M332" s="22"/>
       <c r="N332" s="4"/>
-      <c r="O332" s="30"/>
       <c r="T332" s="9"/>
       <c r="U332" s="4"/>
       <c r="Z332" s="9"/>
@@ -5179,7 +4844,6 @@
       <c r="L333" s="20"/>
       <c r="M333" s="22"/>
       <c r="N333" s="4"/>
-      <c r="O333" s="30"/>
       <c r="T333" s="9"/>
       <c r="U333" s="4"/>
       <c r="Z333" s="9"/>
@@ -5190,7 +4854,6 @@
       <c r="L334" s="20"/>
       <c r="M334" s="22"/>
       <c r="N334" s="4"/>
-      <c r="O334" s="30"/>
       <c r="T334" s="9"/>
       <c r="U334" s="4"/>
       <c r="Z334" s="9"/>
@@ -5201,7 +4864,6 @@
       <c r="L335" s="20"/>
       <c r="M335" s="22"/>
       <c r="N335" s="4"/>
-      <c r="O335" s="30"/>
       <c r="T335" s="9"/>
       <c r="U335" s="4"/>
       <c r="Z335" s="9"/>
@@ -5212,7 +4874,6 @@
       <c r="L336" s="20"/>
       <c r="M336" s="22"/>
       <c r="N336" s="4"/>
-      <c r="O336" s="30"/>
       <c r="T336" s="9"/>
       <c r="U336" s="4"/>
       <c r="Z336" s="9"/>
@@ -5223,7 +4884,6 @@
       <c r="L337" s="20"/>
       <c r="M337" s="22"/>
       <c r="N337" s="4"/>
-      <c r="O337" s="30"/>
       <c r="T337" s="9"/>
       <c r="U337" s="4"/>
       <c r="Z337" s="9"/>
@@ -5234,7 +4894,6 @@
       <c r="L338" s="20"/>
       <c r="M338" s="22"/>
       <c r="N338" s="4"/>
-      <c r="O338" s="30"/>
       <c r="T338" s="9"/>
       <c r="U338" s="4"/>
       <c r="Z338" s="9"/>
@@ -5245,7 +4904,6 @@
       <c r="L339" s="20"/>
       <c r="M339" s="22"/>
       <c r="N339" s="4"/>
-      <c r="O339" s="30"/>
       <c r="T339" s="9"/>
       <c r="U339" s="4"/>
       <c r="Z339" s="9"/>
@@ -5256,7 +4914,6 @@
       <c r="L340" s="20"/>
       <c r="M340" s="22"/>
       <c r="N340" s="4"/>
-      <c r="O340" s="30"/>
       <c r="T340" s="9"/>
       <c r="U340" s="4"/>
       <c r="Z340" s="9"/>
@@ -5267,7 +4924,6 @@
       <c r="L341" s="20"/>
       <c r="M341" s="22"/>
       <c r="N341" s="4"/>
-      <c r="O341" s="30"/>
       <c r="T341" s="9"/>
       <c r="U341" s="4"/>
       <c r="Z341" s="9"/>
@@ -5278,7 +4934,6 @@
       <c r="L342" s="20"/>
       <c r="M342" s="22"/>
       <c r="N342" s="4"/>
-      <c r="O342" s="30"/>
       <c r="T342" s="9"/>
       <c r="U342" s="4"/>
       <c r="Z342" s="9"/>
@@ -5289,7 +4944,6 @@
       <c r="L343" s="20"/>
       <c r="M343" s="22"/>
       <c r="N343" s="4"/>
-      <c r="O343" s="30"/>
       <c r="T343" s="9"/>
       <c r="U343" s="4"/>
       <c r="Z343" s="9"/>
@@ -5300,7 +4954,6 @@
       <c r="L344" s="20"/>
       <c r="M344" s="22"/>
       <c r="N344" s="4"/>
-      <c r="O344" s="30"/>
       <c r="T344" s="9"/>
       <c r="U344" s="4"/>
       <c r="Z344" s="9"/>
@@ -5311,7 +4964,6 @@
       <c r="L345" s="20"/>
       <c r="M345" s="22"/>
       <c r="N345" s="4"/>
-      <c r="O345" s="30"/>
       <c r="T345" s="9"/>
       <c r="U345" s="4"/>
       <c r="Z345" s="9"/>
@@ -5322,7 +4974,6 @@
       <c r="L346" s="20"/>
       <c r="M346" s="22"/>
       <c r="N346" s="4"/>
-      <c r="O346" s="30"/>
       <c r="T346" s="9"/>
       <c r="U346" s="4"/>
       <c r="Z346" s="9"/>
@@ -5333,7 +4984,6 @@
       <c r="L347" s="20"/>
       <c r="M347" s="22"/>
       <c r="N347" s="4"/>
-      <c r="O347" s="30"/>
       <c r="T347" s="9"/>
       <c r="U347" s="4"/>
       <c r="Z347" s="9"/>
@@ -5344,7 +4994,6 @@
       <c r="L348" s="20"/>
       <c r="M348" s="22"/>
       <c r="N348" s="4"/>
-      <c r="O348" s="30"/>
       <c r="T348" s="9"/>
       <c r="U348" s="4"/>
       <c r="Z348" s="9"/>
@@ -5355,7 +5004,6 @@
       <c r="L349" s="20"/>
       <c r="M349" s="22"/>
       <c r="N349" s="4"/>
-      <c r="O349" s="30"/>
       <c r="T349" s="9"/>
       <c r="U349" s="4"/>
       <c r="Z349" s="9"/>
@@ -5366,7 +5014,6 @@
       <c r="L350" s="20"/>
       <c r="M350" s="22"/>
       <c r="N350" s="4"/>
-      <c r="O350" s="30"/>
       <c r="T350" s="9"/>
       <c r="U350" s="4"/>
       <c r="Z350" s="9"/>
@@ -5377,7 +5024,6 @@
       <c r="L351" s="20"/>
       <c r="M351" s="22"/>
       <c r="N351" s="4"/>
-      <c r="O351" s="30"/>
       <c r="T351" s="9"/>
       <c r="U351" s="4"/>
       <c r="Z351" s="9"/>
@@ -5388,7 +5034,6 @@
       <c r="L352" s="20"/>
       <c r="M352" s="22"/>
       <c r="N352" s="4"/>
-      <c r="O352" s="30"/>
       <c r="T352" s="9"/>
       <c r="U352" s="4"/>
       <c r="Z352" s="9"/>
@@ -5399,7 +5044,6 @@
       <c r="L353" s="20"/>
       <c r="M353" s="22"/>
       <c r="N353" s="4"/>
-      <c r="O353" s="30"/>
       <c r="T353" s="9"/>
       <c r="U353" s="4"/>
       <c r="Z353" s="9"/>
@@ -5410,7 +5054,6 @@
       <c r="L354" s="20"/>
       <c r="M354" s="22"/>
       <c r="N354" s="4"/>
-      <c r="O354" s="30"/>
       <c r="T354" s="9"/>
       <c r="U354" s="4"/>
       <c r="Z354" s="9"/>
@@ -5421,7 +5064,6 @@
       <c r="L355" s="20"/>
       <c r="M355" s="22"/>
       <c r="N355" s="4"/>
-      <c r="O355" s="30"/>
       <c r="T355" s="9"/>
       <c r="U355" s="4"/>
       <c r="Z355" s="9"/>
@@ -5432,7 +5074,6 @@
       <c r="L356" s="20"/>
       <c r="M356" s="22"/>
       <c r="N356" s="4"/>
-      <c r="O356" s="30"/>
       <c r="T356" s="9"/>
       <c r="U356" s="4"/>
       <c r="Z356" s="9"/>
@@ -5443,7 +5084,6 @@
       <c r="L357" s="20"/>
       <c r="M357" s="22"/>
       <c r="N357" s="4"/>
-      <c r="O357" s="30"/>
       <c r="T357" s="9"/>
       <c r="U357" s="4"/>
       <c r="Z357" s="9"/>
@@ -5454,7 +5094,6 @@
       <c r="L358" s="20"/>
       <c r="M358" s="22"/>
       <c r="N358" s="4"/>
-      <c r="O358" s="30"/>
       <c r="T358" s="9"/>
       <c r="U358" s="4"/>
       <c r="Z358" s="9"/>
@@ -5465,7 +5104,6 @@
       <c r="L359" s="20"/>
       <c r="M359" s="22"/>
       <c r="N359" s="4"/>
-      <c r="O359" s="30"/>
       <c r="T359" s="9"/>
       <c r="U359" s="4"/>
       <c r="Z359" s="9"/>
@@ -5476,7 +5114,6 @@
       <c r="L360" s="20"/>
       <c r="M360" s="22"/>
       <c r="N360" s="4"/>
-      <c r="O360" s="30"/>
       <c r="T360" s="9"/>
       <c r="U360" s="4"/>
       <c r="Z360" s="9"/>
@@ -5487,7 +5124,6 @@
       <c r="L361" s="20"/>
       <c r="M361" s="22"/>
       <c r="N361" s="4"/>
-      <c r="O361" s="30"/>
       <c r="T361" s="9"/>
       <c r="U361" s="4"/>
       <c r="Z361" s="9"/>
@@ -5498,7 +5134,6 @@
       <c r="L362" s="20"/>
       <c r="M362" s="22"/>
       <c r="N362" s="4"/>
-      <c r="O362" s="30"/>
       <c r="T362" s="9"/>
       <c r="U362" s="4"/>
       <c r="Z362" s="9"/>
@@ -5509,7 +5144,6 @@
       <c r="L363" s="20"/>
       <c r="M363" s="22"/>
       <c r="N363" s="4"/>
-      <c r="O363" s="30"/>
       <c r="T363" s="9"/>
       <c r="U363" s="4"/>
       <c r="Z363" s="9"/>
@@ -5520,7 +5154,6 @@
       <c r="L364" s="20"/>
       <c r="M364" s="22"/>
       <c r="N364" s="4"/>
-      <c r="O364" s="30"/>
       <c r="T364" s="9"/>
       <c r="U364" s="4"/>
       <c r="Z364" s="9"/>
@@ -5531,7 +5164,6 @@
       <c r="L365" s="20"/>
       <c r="M365" s="22"/>
       <c r="N365" s="4"/>
-      <c r="O365" s="30"/>
       <c r="T365" s="9"/>
       <c r="U365" s="4"/>
       <c r="Z365" s="9"/>
@@ -5542,7 +5174,6 @@
       <c r="L366" s="20"/>
       <c r="M366" s="22"/>
       <c r="N366" s="4"/>
-      <c r="O366" s="30"/>
       <c r="T366" s="9"/>
       <c r="U366" s="4"/>
       <c r="Z366" s="9"/>
@@ -5553,7 +5184,6 @@
       <c r="L367" s="20"/>
       <c r="M367" s="22"/>
       <c r="N367" s="4"/>
-      <c r="O367" s="30"/>
       <c r="T367" s="9"/>
       <c r="U367" s="4"/>
       <c r="Z367" s="9"/>
@@ -5564,7 +5194,6 @@
       <c r="L368" s="20"/>
       <c r="M368" s="22"/>
       <c r="N368" s="4"/>
-      <c r="O368" s="30"/>
       <c r="T368" s="9"/>
       <c r="U368" s="4"/>
       <c r="Z368" s="9"/>
@@ -5575,7 +5204,6 @@
       <c r="L369" s="20"/>
       <c r="M369" s="22"/>
       <c r="N369" s="4"/>
-      <c r="O369" s="30"/>
       <c r="T369" s="9"/>
       <c r="U369" s="4"/>
       <c r="Z369" s="9"/>
@@ -5586,7 +5214,6 @@
       <c r="L370" s="20"/>
       <c r="M370" s="22"/>
       <c r="N370" s="4"/>
-      <c r="O370" s="30"/>
       <c r="T370" s="9"/>
       <c r="U370" s="4"/>
       <c r="Z370" s="9"/>
@@ -5597,7 +5224,6 @@
       <c r="L371" s="20"/>
       <c r="M371" s="22"/>
       <c r="N371" s="4"/>
-      <c r="O371" s="30"/>
       <c r="T371" s="9"/>
       <c r="U371" s="4"/>
       <c r="Z371" s="9"/>
@@ -5608,7 +5234,6 @@
       <c r="L372" s="20"/>
       <c r="M372" s="22"/>
       <c r="N372" s="4"/>
-      <c r="O372" s="30"/>
       <c r="T372" s="9"/>
       <c r="U372" s="4"/>
       <c r="Z372" s="9"/>
@@ -5619,7 +5244,6 @@
       <c r="L373" s="20"/>
       <c r="M373" s="22"/>
       <c r="N373" s="4"/>
-      <c r="O373" s="30"/>
       <c r="T373" s="9"/>
       <c r="U373" s="4"/>
       <c r="Z373" s="9"/>
@@ -5630,7 +5254,6 @@
       <c r="L374" s="20"/>
       <c r="M374" s="22"/>
       <c r="N374" s="4"/>
-      <c r="O374" s="30"/>
       <c r="T374" s="9"/>
       <c r="U374" s="4"/>
       <c r="Z374" s="9"/>
@@ -5641,7 +5264,6 @@
       <c r="L375" s="20"/>
       <c r="M375" s="22"/>
       <c r="N375" s="4"/>
-      <c r="O375" s="30"/>
       <c r="T375" s="9"/>
       <c r="U375" s="4"/>
       <c r="Z375" s="9"/>
@@ -5652,7 +5274,6 @@
       <c r="L376" s="20"/>
       <c r="M376" s="22"/>
       <c r="N376" s="4"/>
-      <c r="O376" s="30"/>
       <c r="T376" s="9"/>
       <c r="U376" s="4"/>
       <c r="Z376" s="9"/>
@@ -5663,7 +5284,6 @@
       <c r="L377" s="20"/>
       <c r="M377" s="22"/>
       <c r="N377" s="4"/>
-      <c r="O377" s="30"/>
       <c r="T377" s="9"/>
       <c r="U377" s="4"/>
       <c r="Z377" s="9"/>
@@ -5674,7 +5294,6 @@
       <c r="L378" s="20"/>
       <c r="M378" s="22"/>
       <c r="N378" s="4"/>
-      <c r="O378" s="30"/>
       <c r="T378" s="9"/>
       <c r="U378" s="4"/>
       <c r="Z378" s="9"/>
@@ -5685,7 +5304,6 @@
       <c r="L379" s="20"/>
       <c r="M379" s="22"/>
       <c r="N379" s="4"/>
-      <c r="O379" s="30"/>
       <c r="T379" s="9"/>
       <c r="U379" s="4"/>
       <c r="Z379" s="9"/>
@@ -5696,7 +5314,6 @@
       <c r="L380" s="20"/>
       <c r="M380" s="22"/>
       <c r="N380" s="4"/>
-      <c r="O380" s="30"/>
       <c r="T380" s="9"/>
       <c r="U380" s="4"/>
       <c r="Z380" s="9"/>
@@ -5707,7 +5324,6 @@
       <c r="L381" s="20"/>
       <c r="M381" s="22"/>
       <c r="N381" s="4"/>
-      <c r="O381" s="30"/>
       <c r="T381" s="9"/>
       <c r="U381" s="4"/>
       <c r="Z381" s="9"/>
@@ -5718,7 +5334,6 @@
       <c r="L382" s="20"/>
       <c r="M382" s="22"/>
       <c r="N382" s="4"/>
-      <c r="O382" s="30"/>
       <c r="T382" s="9"/>
       <c r="U382" s="4"/>
       <c r="Z382" s="9"/>
@@ -5729,7 +5344,6 @@
       <c r="L383" s="20"/>
       <c r="M383" s="22"/>
       <c r="N383" s="4"/>
-      <c r="O383" s="30"/>
       <c r="T383" s="9"/>
       <c r="U383" s="4"/>
       <c r="Z383" s="9"/>
@@ -5740,7 +5354,6 @@
       <c r="L384" s="20"/>
       <c r="M384" s="22"/>
       <c r="N384" s="4"/>
-      <c r="O384" s="30"/>
       <c r="T384" s="9"/>
       <c r="U384" s="4"/>
       <c r="Z384" s="9"/>
@@ -5751,7 +5364,6 @@
       <c r="L385" s="20"/>
       <c r="M385" s="22"/>
       <c r="N385" s="4"/>
-      <c r="O385" s="30"/>
       <c r="T385" s="9"/>
       <c r="U385" s="4"/>
       <c r="Z385" s="9"/>
@@ -5762,7 +5374,6 @@
       <c r="L386" s="20"/>
       <c r="M386" s="22"/>
       <c r="N386" s="4"/>
-      <c r="O386" s="30"/>
       <c r="T386" s="9"/>
       <c r="U386" s="4"/>
       <c r="Z386" s="9"/>
@@ -5773,7 +5384,6 @@
       <c r="L387" s="20"/>
       <c r="M387" s="22"/>
       <c r="N387" s="4"/>
-      <c r="O387" s="30"/>
       <c r="T387" s="9"/>
       <c r="U387" s="4"/>
       <c r="Z387" s="9"/>
@@ -5784,7 +5394,6 @@
       <c r="L388" s="20"/>
       <c r="M388" s="22"/>
       <c r="N388" s="4"/>
-      <c r="O388" s="30"/>
       <c r="T388" s="9"/>
       <c r="U388" s="4"/>
       <c r="Z388" s="9"/>
@@ -5795,7 +5404,6 @@
       <c r="L389" s="20"/>
       <c r="M389" s="22"/>
       <c r="N389" s="4"/>
-      <c r="O389" s="30"/>
       <c r="T389" s="9"/>
       <c r="U389" s="4"/>
       <c r="Z389" s="9"/>
@@ -5806,7 +5414,6 @@
       <c r="L390" s="20"/>
       <c r="M390" s="22"/>
       <c r="N390" s="4"/>
-      <c r="O390" s="30"/>
       <c r="T390" s="9"/>
       <c r="U390" s="4"/>
       <c r="Z390" s="9"/>
@@ -5817,7 +5424,6 @@
       <c r="L391" s="20"/>
       <c r="M391" s="22"/>
       <c r="N391" s="4"/>
-      <c r="O391" s="30"/>
       <c r="T391" s="9"/>
       <c r="U391" s="4"/>
       <c r="Z391" s="9"/>
@@ -5828,7 +5434,6 @@
       <c r="L392" s="20"/>
       <c r="M392" s="22"/>
       <c r="N392" s="4"/>
-      <c r="O392" s="30"/>
       <c r="T392" s="9"/>
       <c r="U392" s="4"/>
       <c r="Z392" s="9"/>
@@ -5839,7 +5444,6 @@
       <c r="L393" s="20"/>
       <c r="M393" s="22"/>
       <c r="N393" s="4"/>
-      <c r="O393" s="30"/>
       <c r="T393" s="9"/>
       <c r="U393" s="4"/>
       <c r="Z393" s="9"/>
@@ -5850,7 +5454,6 @@
       <c r="L394" s="20"/>
       <c r="M394" s="22"/>
       <c r="N394" s="4"/>
-      <c r="O394" s="30"/>
       <c r="T394" s="9"/>
       <c r="U394" s="4"/>
       <c r="Z394" s="9"/>
@@ -5861,7 +5464,6 @@
       <c r="L395" s="20"/>
       <c r="M395" s="22"/>
       <c r="N395" s="4"/>
-      <c r="O395" s="30"/>
       <c r="T395" s="9"/>
       <c r="U395" s="4"/>
       <c r="Z395" s="9"/>
@@ -5872,7 +5474,6 @@
       <c r="L396" s="20"/>
       <c r="M396" s="22"/>
       <c r="N396" s="4"/>
-      <c r="O396" s="30"/>
       <c r="T396" s="9"/>
       <c r="U396" s="4"/>
       <c r="Z396" s="9"/>
@@ -5883,7 +5484,6 @@
       <c r="L397" s="20"/>
       <c r="M397" s="22"/>
       <c r="N397" s="4"/>
-      <c r="O397" s="30"/>
       <c r="T397" s="9"/>
       <c r="U397" s="4"/>
       <c r="Z397" s="9"/>
@@ -5894,7 +5494,6 @@
       <c r="L398" s="20"/>
       <c r="M398" s="22"/>
       <c r="N398" s="4"/>
-      <c r="O398" s="30"/>
       <c r="T398" s="9"/>
       <c r="U398" s="4"/>
       <c r="Z398" s="9"/>
@@ -5905,7 +5504,6 @@
       <c r="L399" s="20"/>
       <c r="M399" s="22"/>
       <c r="N399" s="4"/>
-      <c r="O399" s="30"/>
       <c r="T399" s="9"/>
       <c r="U399" s="4"/>
       <c r="Z399" s="9"/>
@@ -5916,7 +5514,6 @@
       <c r="L400" s="20"/>
       <c r="M400" s="22"/>
       <c r="N400" s="4"/>
-      <c r="O400" s="30"/>
       <c r="T400" s="9"/>
       <c r="U400" s="4"/>
       <c r="Z400" s="9"/>
@@ -5927,7 +5524,6 @@
       <c r="L401" s="20"/>
       <c r="M401" s="22"/>
       <c r="N401" s="4"/>
-      <c r="O401" s="30"/>
       <c r="T401" s="9"/>
       <c r="U401" s="4"/>
       <c r="Z401" s="9"/>
@@ -5938,7 +5534,6 @@
       <c r="L402" s="20"/>
       <c r="M402" s="22"/>
       <c r="N402" s="4"/>
-      <c r="O402" s="30"/>
       <c r="T402" s="9"/>
       <c r="U402" s="4"/>
       <c r="Z402" s="9"/>
@@ -5949,7 +5544,6 @@
       <c r="L403" s="20"/>
       <c r="M403" s="22"/>
       <c r="N403" s="4"/>
-      <c r="O403" s="30"/>
       <c r="T403" s="9"/>
       <c r="U403" s="4"/>
       <c r="Z403" s="9"/>
@@ -5960,7 +5554,6 @@
       <c r="L404" s="20"/>
       <c r="M404" s="22"/>
       <c r="N404" s="4"/>
-      <c r="O404" s="30"/>
       <c r="T404" s="9"/>
       <c r="U404" s="4"/>
       <c r="Z404" s="9"/>
@@ -5971,7 +5564,6 @@
       <c r="L405" s="20"/>
       <c r="M405" s="22"/>
       <c r="N405" s="4"/>
-      <c r="O405" s="30"/>
       <c r="T405" s="9"/>
       <c r="U405" s="4"/>
       <c r="Z405" s="9"/>
@@ -5982,7 +5574,6 @@
       <c r="L406" s="20"/>
       <c r="M406" s="22"/>
       <c r="N406" s="4"/>
-      <c r="O406" s="30"/>
       <c r="T406" s="9"/>
       <c r="U406" s="4"/>
       <c r="Z406" s="9"/>
@@ -5993,7 +5584,6 @@
       <c r="L407" s="20"/>
       <c r="M407" s="22"/>
       <c r="N407" s="4"/>
-      <c r="O407" s="30"/>
       <c r="T407" s="9"/>
       <c r="U407" s="4"/>
       <c r="Z407" s="9"/>
@@ -6004,7 +5594,6 @@
       <c r="L408" s="20"/>
       <c r="M408" s="22"/>
       <c r="N408" s="4"/>
-      <c r="O408" s="30"/>
       <c r="T408" s="9"/>
       <c r="U408" s="4"/>
       <c r="Z408" s="9"/>
@@ -6015,7 +5604,6 @@
       <c r="L409" s="20"/>
       <c r="M409" s="22"/>
       <c r="N409" s="4"/>
-      <c r="O409" s="30"/>
       <c r="T409" s="9"/>
       <c r="U409" s="4"/>
       <c r="Z409" s="9"/>
@@ -6026,7 +5614,6 @@
       <c r="L410" s="20"/>
       <c r="M410" s="22"/>
       <c r="N410" s="4"/>
-      <c r="O410" s="30"/>
       <c r="T410" s="9"/>
       <c r="U410" s="4"/>
       <c r="Z410" s="9"/>
@@ -6037,7 +5624,6 @@
       <c r="L411" s="20"/>
       <c r="M411" s="22"/>
       <c r="N411" s="4"/>
-      <c r="O411" s="30"/>
       <c r="T411" s="9"/>
       <c r="U411" s="4"/>
       <c r="Z411" s="9"/>
@@ -6048,7 +5634,6 @@
       <c r="L412" s="20"/>
       <c r="M412" s="22"/>
       <c r="N412" s="4"/>
-      <c r="O412" s="30"/>
       <c r="T412" s="9"/>
       <c r="U412" s="4"/>
       <c r="Z412" s="9"/>
@@ -6059,7 +5644,6 @@
       <c r="L413" s="20"/>
       <c r="M413" s="22"/>
       <c r="N413" s="4"/>
-      <c r="O413" s="30"/>
       <c r="T413" s="9"/>
       <c r="U413" s="4"/>
       <c r="Z413" s="9"/>
@@ -6070,7 +5654,6 @@
       <c r="L414" s="20"/>
       <c r="M414" s="22"/>
       <c r="N414" s="4"/>
-      <c r="O414" s="30"/>
       <c r="T414" s="9"/>
       <c r="U414" s="4"/>
       <c r="Z414" s="9"/>
@@ -6081,7 +5664,6 @@
       <c r="L415" s="20"/>
       <c r="M415" s="22"/>
       <c r="N415" s="4"/>
-      <c r="O415" s="30"/>
       <c r="T415" s="9"/>
       <c r="U415" s="4"/>
       <c r="Z415" s="9"/>
@@ -6092,7 +5674,6 @@
       <c r="L416" s="20"/>
       <c r="M416" s="22"/>
       <c r="N416" s="4"/>
-      <c r="O416" s="30"/>
       <c r="T416" s="9"/>
       <c r="U416" s="4"/>
       <c r="Z416" s="9"/>
@@ -6103,7 +5684,6 @@
       <c r="L417" s="20"/>
       <c r="M417" s="22"/>
       <c r="N417" s="4"/>
-      <c r="O417" s="30"/>
       <c r="T417" s="9"/>
       <c r="U417" s="4"/>
       <c r="Z417" s="9"/>
@@ -6114,7 +5694,6 @@
       <c r="L418" s="20"/>
       <c r="M418" s="22"/>
       <c r="N418" s="4"/>
-      <c r="O418" s="30"/>
       <c r="T418" s="9"/>
       <c r="U418" s="4"/>
       <c r="Z418" s="9"/>
@@ -6125,7 +5704,6 @@
       <c r="L419" s="20"/>
       <c r="M419" s="22"/>
       <c r="N419" s="4"/>
-      <c r="O419" s="30"/>
       <c r="T419" s="9"/>
       <c r="U419" s="4"/>
       <c r="Z419" s="9"/>
@@ -6136,7 +5714,6 @@
       <c r="L420" s="20"/>
       <c r="M420" s="22"/>
       <c r="N420" s="4"/>
-      <c r="O420" s="30"/>
       <c r="T420" s="9"/>
       <c r="U420" s="4"/>
       <c r="Z420" s="9"/>
@@ -6147,7 +5724,6 @@
       <c r="L421" s="20"/>
       <c r="M421" s="22"/>
       <c r="N421" s="4"/>
-      <c r="O421" s="30"/>
       <c r="T421" s="9"/>
       <c r="U421" s="4"/>
       <c r="Z421" s="9"/>
@@ -6158,7 +5734,6 @@
       <c r="L422" s="20"/>
       <c r="M422" s="22"/>
       <c r="N422" s="4"/>
-      <c r="O422" s="30"/>
       <c r="T422" s="9"/>
       <c r="U422" s="4"/>
       <c r="Z422" s="9"/>
@@ -6169,7 +5744,6 @@
       <c r="L423" s="20"/>
       <c r="M423" s="22"/>
       <c r="N423" s="4"/>
-      <c r="O423" s="30"/>
       <c r="T423" s="9"/>
       <c r="U423" s="4"/>
       <c r="Z423" s="9"/>
@@ -6180,7 +5754,6 @@
       <c r="L424" s="20"/>
       <c r="M424" s="22"/>
       <c r="N424" s="4"/>
-      <c r="O424" s="30"/>
       <c r="T424" s="9"/>
       <c r="U424" s="4"/>
       <c r="Z424" s="9"/>
@@ -6191,7 +5764,6 @@
       <c r="L425" s="20"/>
       <c r="M425" s="22"/>
       <c r="N425" s="4"/>
-      <c r="O425" s="30"/>
       <c r="T425" s="9"/>
       <c r="U425" s="4"/>
       <c r="Z425" s="9"/>
@@ -6202,7 +5774,6 @@
       <c r="L426" s="20"/>
       <c r="M426" s="22"/>
       <c r="N426" s="4"/>
-      <c r="O426" s="30"/>
       <c r="T426" s="9"/>
       <c r="U426" s="4"/>
       <c r="Z426" s="9"/>
@@ -6213,7 +5784,6 @@
       <c r="L427" s="20"/>
       <c r="M427" s="22"/>
       <c r="N427" s="4"/>
-      <c r="O427" s="30"/>
       <c r="T427" s="9"/>
       <c r="U427" s="4"/>
       <c r="Z427" s="9"/>
@@ -6224,7 +5794,6 @@
       <c r="L428" s="20"/>
       <c r="M428" s="22"/>
       <c r="N428" s="4"/>
-      <c r="O428" s="30"/>
       <c r="T428" s="9"/>
       <c r="U428" s="4"/>
       <c r="Z428" s="9"/>
@@ -6235,7 +5804,6 @@
       <c r="L429" s="20"/>
       <c r="M429" s="22"/>
       <c r="N429" s="4"/>
-      <c r="O429" s="30"/>
       <c r="T429" s="9"/>
       <c r="U429" s="4"/>
       <c r="Z429" s="9"/>
@@ -6246,7 +5814,6 @@
       <c r="L430" s="20"/>
       <c r="M430" s="22"/>
       <c r="N430" s="4"/>
-      <c r="O430" s="30"/>
       <c r="T430" s="9"/>
       <c r="U430" s="4"/>
       <c r="Z430" s="9"/>
@@ -6257,7 +5824,6 @@
       <c r="L431" s="20"/>
       <c r="M431" s="22"/>
       <c r="N431" s="4"/>
-      <c r="O431" s="30"/>
       <c r="T431" s="9"/>
       <c r="U431" s="4"/>
       <c r="Z431" s="9"/>
@@ -6268,7 +5834,6 @@
       <c r="L432" s="20"/>
       <c r="M432" s="22"/>
       <c r="N432" s="4"/>
-      <c r="O432" s="30"/>
       <c r="T432" s="9"/>
       <c r="U432" s="4"/>
       <c r="Z432" s="9"/>
@@ -6279,7 +5844,6 @@
       <c r="L433" s="20"/>
       <c r="M433" s="22"/>
       <c r="N433" s="4"/>
-      <c r="O433" s="30"/>
       <c r="T433" s="9"/>
       <c r="U433" s="4"/>
       <c r="Z433" s="9"/>
@@ -6290,7 +5854,6 @@
       <c r="L434" s="20"/>
       <c r="M434" s="22"/>
       <c r="N434" s="4"/>
-      <c r="O434" s="30"/>
       <c r="T434" s="9"/>
       <c r="U434" s="4"/>
       <c r="Z434" s="9"/>
@@ -6301,7 +5864,6 @@
       <c r="L435" s="20"/>
       <c r="M435" s="22"/>
       <c r="N435" s="4"/>
-      <c r="O435" s="30"/>
       <c r="T435" s="9"/>
       <c r="U435" s="4"/>
       <c r="Z435" s="9"/>
@@ -6312,7 +5874,6 @@
       <c r="L436" s="20"/>
       <c r="M436" s="22"/>
       <c r="N436" s="4"/>
-      <c r="O436" s="30"/>
       <c r="T436" s="9"/>
       <c r="U436" s="4"/>
       <c r="Z436" s="9"/>
@@ -6323,7 +5884,6 @@
       <c r="L437" s="20"/>
       <c r="M437" s="22"/>
       <c r="N437" s="4"/>
-      <c r="O437" s="30"/>
       <c r="T437" s="9"/>
       <c r="U437" s="4"/>
       <c r="Z437" s="9"/>
@@ -6334,7 +5894,6 @@
       <c r="L438" s="20"/>
       <c r="M438" s="22"/>
       <c r="N438" s="4"/>
-      <c r="O438" s="30"/>
       <c r="T438" s="9"/>
       <c r="U438" s="4"/>
       <c r="Z438" s="9"/>
@@ -6345,7 +5904,6 @@
       <c r="L439" s="20"/>
       <c r="M439" s="22"/>
       <c r="N439" s="4"/>
-      <c r="O439" s="30"/>
       <c r="T439" s="9"/>
       <c r="U439" s="4"/>
       <c r="Z439" s="9"/>
@@ -6356,7 +5914,6 @@
       <c r="L440" s="20"/>
       <c r="M440" s="22"/>
       <c r="N440" s="4"/>
-      <c r="O440" s="30"/>
       <c r="T440" s="9"/>
       <c r="U440" s="4"/>
       <c r="Z440" s="9"/>
@@ -6367,7 +5924,6 @@
       <c r="L441" s="20"/>
       <c r="M441" s="22"/>
       <c r="N441" s="4"/>
-      <c r="O441" s="30"/>
       <c r="T441" s="9"/>
       <c r="U441" s="4"/>
       <c r="Z441" s="9"/>
@@ -6378,7 +5934,6 @@
       <c r="L442" s="20"/>
       <c r="M442" s="22"/>
       <c r="N442" s="4"/>
-      <c r="O442" s="30"/>
       <c r="T442" s="9"/>
       <c r="U442" s="4"/>
       <c r="Z442" s="9"/>
@@ -6389,7 +5944,6 @@
       <c r="L443" s="20"/>
       <c r="M443" s="22"/>
       <c r="N443" s="4"/>
-      <c r="O443" s="30"/>
       <c r="T443" s="9"/>
       <c r="U443" s="4"/>
       <c r="Z443" s="9"/>
@@ -6400,7 +5954,6 @@
       <c r="L444" s="20"/>
       <c r="M444" s="22"/>
       <c r="N444" s="4"/>
-      <c r="O444" s="30"/>
       <c r="T444" s="9"/>
       <c r="U444" s="4"/>
       <c r="Z444" s="9"/>
@@ -6411,7 +5964,6 @@
       <c r="L445" s="20"/>
       <c r="M445" s="22"/>
       <c r="N445" s="4"/>
-      <c r="O445" s="30"/>
       <c r="T445" s="9"/>
       <c r="U445" s="4"/>
       <c r="Z445" s="9"/>
@@ -6422,7 +5974,6 @@
       <c r="L446" s="20"/>
       <c r="M446" s="22"/>
       <c r="N446" s="4"/>
-      <c r="O446" s="30"/>
       <c r="T446" s="9"/>
       <c r="U446" s="4"/>
       <c r="Z446" s="9"/>
@@ -6433,7 +5984,6 @@
       <c r="L447" s="20"/>
       <c r="M447" s="22"/>
       <c r="N447" s="4"/>
-      <c r="O447" s="30"/>
       <c r="T447" s="9"/>
       <c r="U447" s="4"/>
       <c r="Z447" s="9"/>
@@ -6444,7 +5994,6 @@
       <c r="L448" s="20"/>
       <c r="M448" s="22"/>
       <c r="N448" s="4"/>
-      <c r="O448" s="30"/>
       <c r="T448" s="9"/>
       <c r="U448" s="4"/>
       <c r="Z448" s="9"/>
@@ -6455,7 +6004,6 @@
       <c r="L449" s="20"/>
       <c r="M449" s="22"/>
       <c r="N449" s="4"/>
-      <c r="O449" s="30"/>
       <c r="T449" s="9"/>
       <c r="U449" s="4"/>
       <c r="Z449" s="9"/>
@@ -6466,7 +6014,6 @@
       <c r="L450" s="20"/>
       <c r="M450" s="22"/>
       <c r="N450" s="4"/>
-      <c r="O450" s="30"/>
       <c r="T450" s="9"/>
       <c r="U450" s="4"/>
       <c r="Z450" s="9"/>
@@ -6477,7 +6024,6 @@
       <c r="L451" s="20"/>
       <c r="M451" s="22"/>
       <c r="N451" s="4"/>
-      <c r="O451" s="30"/>
       <c r="T451" s="9"/>
       <c r="U451" s="4"/>
       <c r="Z451" s="9"/>
@@ -6488,7 +6034,6 @@
       <c r="L452" s="20"/>
       <c r="M452" s="22"/>
       <c r="N452" s="4"/>
-      <c r="O452" s="30"/>
       <c r="T452" s="9"/>
       <c r="U452" s="4"/>
       <c r="Z452" s="9"/>
@@ -6499,7 +6044,6 @@
       <c r="L453" s="20"/>
       <c r="M453" s="22"/>
       <c r="N453" s="4"/>
-      <c r="O453" s="30"/>
       <c r="T453" s="9"/>
       <c r="U453" s="4"/>
       <c r="Z453" s="9"/>
@@ -6510,7 +6054,6 @@
       <c r="L454" s="20"/>
       <c r="M454" s="22"/>
       <c r="N454" s="4"/>
-      <c r="O454" s="30"/>
       <c r="T454" s="9"/>
       <c r="U454" s="4"/>
       <c r="Z454" s="9"/>
@@ -6521,7 +6064,6 @@
       <c r="L455" s="20"/>
       <c r="M455" s="22"/>
       <c r="N455" s="4"/>
-      <c r="O455" s="30"/>
       <c r="T455" s="9"/>
       <c r="U455" s="4"/>
       <c r="Z455" s="9"/>
@@ -6532,7 +6074,6 @@
       <c r="L456" s="20"/>
       <c r="M456" s="22"/>
       <c r="N456" s="4"/>
-      <c r="O456" s="30"/>
       <c r="T456" s="9"/>
       <c r="U456" s="4"/>
       <c r="Z456" s="9"/>
@@ -6543,7 +6084,6 @@
       <c r="L457" s="20"/>
       <c r="M457" s="22"/>
       <c r="N457" s="4"/>
-      <c r="O457" s="30"/>
       <c r="T457" s="9"/>
       <c r="U457" s="4"/>
       <c r="Z457" s="9"/>
@@ -6554,7 +6094,6 @@
       <c r="L458" s="20"/>
       <c r="M458" s="22"/>
       <c r="N458" s="4"/>
-      <c r="O458" s="30"/>
       <c r="T458" s="9"/>
       <c r="U458" s="4"/>
       <c r="Z458" s="9"/>
@@ -6565,7 +6104,6 @@
       <c r="L459" s="20"/>
       <c r="M459" s="22"/>
       <c r="N459" s="4"/>
-      <c r="O459" s="30"/>
       <c r="T459" s="9"/>
       <c r="U459" s="4"/>
       <c r="Z459" s="9"/>
@@ -6576,7 +6114,6 @@
       <c r="L460" s="20"/>
       <c r="M460" s="22"/>
       <c r="N460" s="4"/>
-      <c r="O460" s="30"/>
       <c r="T460" s="9"/>
       <c r="U460" s="4"/>
       <c r="Z460" s="9"/>
@@ -6587,7 +6124,6 @@
       <c r="L461" s="20"/>
       <c r="M461" s="22"/>
       <c r="N461" s="4"/>
-      <c r="O461" s="30"/>
       <c r="T461" s="9"/>
       <c r="U461" s="4"/>
       <c r="Z461" s="9"/>
@@ -6598,7 +6134,6 @@
       <c r="L462" s="20"/>
       <c r="M462" s="22"/>
       <c r="N462" s="4"/>
-      <c r="O462" s="30"/>
       <c r="T462" s="9"/>
       <c r="U462" s="4"/>
       <c r="Z462" s="9"/>
@@ -6609,7 +6144,6 @@
       <c r="L463" s="20"/>
       <c r="M463" s="22"/>
       <c r="N463" s="4"/>
-      <c r="O463" s="30"/>
       <c r="T463" s="9"/>
       <c r="U463" s="4"/>
       <c r="Z463" s="9"/>
@@ -6620,7 +6154,6 @@
       <c r="L464" s="20"/>
       <c r="M464" s="22"/>
       <c r="N464" s="4"/>
-      <c r="O464" s="30"/>
       <c r="T464" s="9"/>
       <c r="U464" s="4"/>
       <c r="Z464" s="9"/>
@@ -6631,7 +6164,6 @@
       <c r="L465" s="20"/>
       <c r="M465" s="22"/>
       <c r="N465" s="4"/>
-      <c r="O465" s="30"/>
       <c r="T465" s="9"/>
       <c r="U465" s="4"/>
       <c r="Z465" s="9"/>
@@ -6642,7 +6174,6 @@
       <c r="L466" s="20"/>
       <c r="M466" s="22"/>
       <c r="N466" s="4"/>
-      <c r="O466" s="30"/>
       <c r="T466" s="9"/>
       <c r="U466" s="4"/>
       <c r="Z466" s="9"/>
@@ -6653,7 +6184,6 @@
       <c r="L467" s="20"/>
       <c r="M467" s="22"/>
       <c r="N467" s="4"/>
-      <c r="O467" s="30"/>
       <c r="T467" s="9"/>
       <c r="U467" s="4"/>
       <c r="Z467" s="9"/>
@@ -6664,7 +6194,6 @@
       <c r="L468" s="20"/>
       <c r="M468" s="22"/>
       <c r="N468" s="4"/>
-      <c r="O468" s="30"/>
       <c r="T468" s="9"/>
       <c r="U468" s="4"/>
       <c r="Z468" s="9"/>
@@ -6675,7 +6204,6 @@
       <c r="L469" s="20"/>
       <c r="M469" s="22"/>
       <c r="N469" s="4"/>
-      <c r="O469" s="30"/>
       <c r="T469" s="9"/>
       <c r="U469" s="4"/>
       <c r="Z469" s="9"/>
@@ -6686,7 +6214,6 @@
       <c r="L470" s="20"/>
       <c r="M470" s="22"/>
       <c r="N470" s="4"/>
-      <c r="O470" s="30"/>
       <c r="T470" s="9"/>
       <c r="U470" s="4"/>
       <c r="Z470" s="9"/>
@@ -6697,7 +6224,6 @@
       <c r="L471" s="20"/>
       <c r="M471" s="22"/>
       <c r="N471" s="4"/>
-      <c r="O471" s="30"/>
       <c r="T471" s="9"/>
       <c r="U471" s="4"/>
       <c r="Z471" s="9"/>
@@ -6708,7 +6234,6 @@
       <c r="L472" s="20"/>
       <c r="M472" s="22"/>
       <c r="N472" s="4"/>
-      <c r="O472" s="30"/>
       <c r="T472" s="9"/>
       <c r="U472" s="4"/>
       <c r="Z472" s="9"/>
@@ -6719,7 +6244,6 @@
       <c r="L473" s="20"/>
       <c r="M473" s="22"/>
       <c r="N473" s="4"/>
-      <c r="O473" s="30"/>
       <c r="T473" s="9"/>
       <c r="U473" s="4"/>
       <c r="Z473" s="9"/>
@@ -6730,7 +6254,6 @@
       <c r="L474" s="20"/>
       <c r="M474" s="22"/>
       <c r="N474" s="4"/>
-      <c r="O474" s="30"/>
       <c r="T474" s="9"/>
       <c r="U474" s="4"/>
       <c r="Z474" s="9"/>
@@ -6741,7 +6264,6 @@
       <c r="L475" s="20"/>
       <c r="M475" s="22"/>
       <c r="N475" s="4"/>
-      <c r="O475" s="30"/>
       <c r="T475" s="9"/>
       <c r="U475" s="4"/>
       <c r="Z475" s="9"/>
@@ -6752,7 +6274,6 @@
       <c r="L476" s="20"/>
       <c r="M476" s="22"/>
       <c r="N476" s="4"/>
-      <c r="O476" s="30"/>
       <c r="T476" s="9"/>
       <c r="U476" s="4"/>
       <c r="Z476" s="9"/>
@@ -6763,7 +6284,6 @@
       <c r="L477" s="20"/>
       <c r="M477" s="22"/>
       <c r="N477" s="4"/>
-      <c r="O477" s="30"/>
       <c r="T477" s="9"/>
       <c r="U477" s="4"/>
       <c r="Z477" s="9"/>
@@ -6774,7 +6294,6 @@
       <c r="L478" s="20"/>
       <c r="M478" s="22"/>
       <c r="N478" s="4"/>
-      <c r="O478" s="30"/>
       <c r="T478" s="9"/>
       <c r="U478" s="4"/>
       <c r="Z478" s="9"/>
@@ -6785,7 +6304,6 @@
       <c r="L479" s="20"/>
       <c r="M479" s="22"/>
       <c r="N479" s="4"/>
-      <c r="O479" s="30"/>
       <c r="T479" s="9"/>
       <c r="U479" s="4"/>
       <c r="Z479" s="9"/>
@@ -6796,7 +6314,6 @@
       <c r="L480" s="20"/>
       <c r="M480" s="22"/>
       <c r="N480" s="4"/>
-      <c r="O480" s="30"/>
       <c r="T480" s="9"/>
       <c r="U480" s="4"/>
       <c r="Z480" s="9"/>
@@ -6807,7 +6324,6 @@
       <c r="L481" s="20"/>
       <c r="M481" s="22"/>
       <c r="N481" s="4"/>
-      <c r="O481" s="30"/>
       <c r="T481" s="9"/>
       <c r="U481" s="4"/>
       <c r="Z481" s="9"/>
@@ -6818,7 +6334,6 @@
       <c r="L482" s="20"/>
       <c r="M482" s="22"/>
       <c r="N482" s="4"/>
-      <c r="O482" s="30"/>
       <c r="T482" s="9"/>
       <c r="U482" s="4"/>
       <c r="Z482" s="9"/>
@@ -6829,7 +6344,6 @@
       <c r="L483" s="20"/>
       <c r="M483" s="22"/>
       <c r="N483" s="4"/>
-      <c r="O483" s="30"/>
       <c r="T483" s="9"/>
       <c r="U483" s="4"/>
       <c r="Z483" s="9"/>
@@ -6840,7 +6354,6 @@
       <c r="L484" s="20"/>
       <c r="M484" s="22"/>
       <c r="N484" s="4"/>
-      <c r="O484" s="30"/>
       <c r="T484" s="9"/>
       <c r="U484" s="4"/>
       <c r="Z484" s="9"/>
@@ -6851,7 +6364,6 @@
       <c r="L485" s="20"/>
       <c r="M485" s="22"/>
       <c r="N485" s="4"/>
-      <c r="O485" s="30"/>
       <c r="T485" s="9"/>
       <c r="U485" s="4"/>
       <c r="Z485" s="9"/>
@@ -6862,7 +6374,6 @@
       <c r="L486" s="20"/>
       <c r="M486" s="22"/>
       <c r="N486" s="4"/>
-      <c r="O486" s="30"/>
       <c r="T486" s="9"/>
       <c r="U486" s="4"/>
       <c r="Z486" s="9"/>
@@ -6873,7 +6384,6 @@
       <c r="L487" s="20"/>
       <c r="M487" s="22"/>
       <c r="N487" s="4"/>
-      <c r="O487" s="30"/>
       <c r="T487" s="9"/>
       <c r="U487" s="4"/>
       <c r="Z487" s="9"/>
@@ -6884,7 +6394,6 @@
       <c r="L488" s="20"/>
       <c r="M488" s="22"/>
       <c r="N488" s="4"/>
-      <c r="O488" s="30"/>
       <c r="T488" s="9"/>
       <c r="U488" s="4"/>
       <c r="Z488" s="9"/>
@@ -6895,7 +6404,6 @@
       <c r="L489" s="20"/>
       <c r="M489" s="22"/>
       <c r="N489" s="4"/>
-      <c r="O489" s="30"/>
       <c r="T489" s="9"/>
       <c r="U489" s="4"/>
       <c r="Z489" s="9"/>
@@ -6906,7 +6414,6 @@
       <c r="L490" s="20"/>
       <c r="M490" s="22"/>
       <c r="N490" s="4"/>
-      <c r="O490" s="30"/>
       <c r="T490" s="9"/>
       <c r="U490" s="4"/>
       <c r="Z490" s="9"/>
@@ -6917,7 +6424,6 @@
       <c r="L491" s="20"/>
       <c r="M491" s="22"/>
       <c r="N491" s="4"/>
-      <c r="O491" s="30"/>
       <c r="T491" s="9"/>
       <c r="U491" s="4"/>
       <c r="Z491" s="9"/>
@@ -6928,7 +6434,6 @@
       <c r="L492" s="20"/>
       <c r="M492" s="22"/>
       <c r="N492" s="4"/>
-      <c r="O492" s="30"/>
       <c r="T492" s="9"/>
       <c r="U492" s="4"/>
       <c r="Z492" s="9"/>
@@ -6939,7 +6444,6 @@
       <c r="L493" s="20"/>
       <c r="M493" s="22"/>
       <c r="N493" s="4"/>
-      <c r="O493" s="30"/>
       <c r="T493" s="9"/>
       <c r="U493" s="4"/>
       <c r="Z493" s="9"/>
@@ -6950,7 +6454,6 @@
       <c r="L494" s="20"/>
       <c r="M494" s="22"/>
       <c r="N494" s="4"/>
-      <c r="O494" s="30"/>
       <c r="T494" s="9"/>
       <c r="U494" s="4"/>
       <c r="Z494" s="9"/>
@@ -6961,7 +6464,6 @@
       <c r="L495" s="20"/>
       <c r="M495" s="22"/>
       <c r="N495" s="4"/>
-      <c r="O495" s="30"/>
       <c r="T495" s="9"/>
       <c r="U495" s="4"/>
       <c r="Z495" s="9"/>
@@ -6972,7 +6474,6 @@
       <c r="L496" s="20"/>
       <c r="M496" s="22"/>
       <c r="N496" s="4"/>
-      <c r="O496" s="30"/>
       <c r="T496" s="9"/>
       <c r="U496" s="4"/>
       <c r="Z496" s="9"/>
@@ -6983,7 +6484,6 @@
       <c r="L497" s="20"/>
       <c r="M497" s="22"/>
       <c r="N497" s="4"/>
-      <c r="O497" s="30"/>
       <c r="T497" s="9"/>
       <c r="U497" s="4"/>
       <c r="Z497" s="9"/>
@@ -6994,7 +6494,6 @@
       <c r="L498" s="20"/>
       <c r="M498" s="22"/>
       <c r="N498" s="4"/>
-      <c r="O498" s="30"/>
       <c r="T498" s="9"/>
       <c r="U498" s="4"/>
       <c r="Z498" s="9"/>
@@ -7005,7 +6504,6 @@
       <c r="L499" s="20"/>
       <c r="M499" s="22"/>
       <c r="N499" s="4"/>
-      <c r="O499" s="30"/>
       <c r="T499" s="9"/>
       <c r="U499" s="4"/>
       <c r="Z499" s="9"/>

</xml_diff>